<commit_message>
AVD roadmap from AVD FY27 Milestones page (10/19)
</commit_message>
<xml_diff>
--- a/data/roadmaps/Roadmap - Combined.xlsx
+++ b/data/roadmaps/Roadmap - Combined.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Area" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Initiatives" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Product Area" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Initiatives" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Milestones" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reference" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Initiatives'!$A$1:$O$201</definedName>
@@ -971,7 +971,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Draft from weekly PO updates (9/16, 9/23, 10/7)</t>
+          <t>Draft from weekly PO updates (9/16, 9/23, 10/7); AVD from AVD FY27 Milestones page (10/19)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>46302</v>
+        <v>46314</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>AVD onboarding process and job codes</t>
+          <t>AVD Operations in a Production Ready State</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
@@ -2524,26 +2524,30 @@
         </is>
       </c>
       <c r="G26" s="15" t="n">
-        <v>46266</v>
+        <v>46274</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>46387</v>
+        <v>46660</v>
       </c>
       <c r="I26" s="13" t="n"/>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>A documented, repeatable way to request and onboard users to AVD, including application job codes.</t>
+          <t>Patching, backup, golden image, CrowdStrike, vulnerability scanning, autoscaling, DR, change management and CCG updates.</t>
         </is>
       </c>
       <c r="K26" s="13" t="n"/>
       <c r="L26" s="13" t="n"/>
-      <c r="M26" s="14" t="n"/>
+      <c r="M26" s="14" t="inlineStr">
+        <is>
+          <t>Patching owner TBD (Citrix patches its own; decide with MiSP). Golden image approach pending with the Citrix team and SecOps. CrowdStrike: CLDSPT-114612 awaiting SecOps feedback. Disaster recovery blocked until the Azure West region is complete. Vulnerability scanning waits on Multi Session Host Pools (AVD-05).</t>
+        </is>
+      </c>
       <c r="N26" s="15" t="n">
-        <v>46302</v>
+        <v>46314</v>
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Met with Citrix team; documented discrepancies; onboarding doc being updated; job code template in progress; Jira request type for AVD added by Agile Tools (9/23); approved for an application ID in BaseCamp (10/7). EOC team to pilot the process. Source: COMET&lt;&gt;CMS PO updates.</t>
+          <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
       </c>
     </row>
@@ -2560,12 +2564,12 @@
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>VDI production hardening</t>
+          <t>AVD End User Support Services Operationalized</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Secure access &amp; compliance</t>
+          <t>Production readiness &amp; operations</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -2579,30 +2583,30 @@
         </is>
       </c>
       <c r="G27" s="15" t="n">
-        <v>46235</v>
+        <v>46259</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>46387</v>
+        <v>46477</v>
       </c>
       <c r="I27" s="13" t="n"/>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>Make the AVD platform production ready: MFA, real-time monitoring, self-restart portal, Zscaler connector, backups and patching.</t>
+          <t>Support model (CLDSPT, EOC, Help Desk, Tier 2, user manual, training) ready for users.</t>
         </is>
       </c>
       <c r="K27" s="13" t="n"/>
       <c r="L27" s="13" t="n"/>
       <c r="M27" s="14" t="inlineStr">
         <is>
-          <t>9/16 and 9/23: REQ0404769 and REQ0404771 escalated for approval. Not listed as blockers on 10/7; confirm they are resolved.</t>
+          <t>Dependencies past their needed-by date: SRE Team EOC workbook items (Datadog integration, alerts, Splunk On-call), needed 8/28; CMS Help Desk / Nerdio CSM KBA approvals, agent trainings and SNOW integration, needed 9/10.</t>
         </is>
       </c>
       <c r="N27" s="15" t="n">
-        <v>46302</v>
+        <v>46314</v>
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Start/end dates are placeholders (not in the updates); confirm with the PO. MFA on Windows App (testing); MFA enrollment off Zscaler in progress; autoscaling done; FSLogix disconnects fixed; self-restart URL avd.cloud.cms.gov (REQ0404769); real-time monitoring (REQ0404771); ZCC Cloud Connector started; GSS backups and patching being set up. Source: COMET&lt;&gt;CMS PO updates.</t>
+          <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
       </c>
     </row>
@@ -2619,12 +2623,12 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>CrowdStrike integration for AVD hosts</t>
+          <t>AVD Onboarding Process Established</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Secure access &amp; compliance</t>
+          <t>Production readiness &amp; operations</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -2638,30 +2642,26 @@
         </is>
       </c>
       <c r="G28" s="15" t="n">
-        <v>46281</v>
+        <v>46266</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>46356</v>
+        <v>46332</v>
       </c>
       <c r="I28" s="13" t="n"/>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>AVD session hosts report to the Falcon console with the right host groups and prevention policies.</t>
-        </is>
-      </c>
-      <c r="K28" s="13" t="inlineStr">
-        <is>
-          <t>CLDSPT-114612</t>
-        </is>
-      </c>
+          <t>Repeatable AVD onboarding: Jira project, ONBI integration, job codes.</t>
+        </is>
+      </c>
+      <c r="K28" s="13" t="n"/>
       <c r="L28" s="13" t="n"/>
       <c r="M28" s="14" t="n"/>
       <c r="N28" s="15" t="n">
-        <v>46302</v>
+        <v>46314</v>
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Only outbound HTTPS (443) needed; next is validating Windows 11 multi-session hosts in the prod subscription. Source: COMET&lt;&gt;CMS PO updates.</t>
+          <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
       </c>
     </row>
@@ -2678,12 +2678,12 @@
       </c>
       <c r="C29" s="14" t="inlineStr">
         <is>
-          <t>AVD support model (EOC, Help Desk T0, Tier 2)</t>
+          <t>VDI User Migrations</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Production readiness &amp; operations</t>
+          <t>Expand hybrid &amp; multi-cloud hosting</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -2697,26 +2697,26 @@
         </is>
       </c>
       <c r="G29" s="15" t="n">
-        <v>46266</v>
+        <v>46391</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>46387</v>
+        <v>46594</v>
       </c>
       <c r="I29" s="13" t="n"/>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>Support path for AVD users: EOC alerting, CMS Help Desk knowledge articles, Cloud Tier 2 and CLDSPT requests.</t>
+          <t>Wave 0 validation (Jan 2027) through Wave 6 (Jul 2027), about 1,045 users combined.</t>
         </is>
       </c>
       <c r="K29" s="13" t="n"/>
       <c r="L29" s="13" t="n"/>
       <c r="M29" s="14" t="n"/>
       <c r="N29" s="15" t="n">
-        <v>46302</v>
+        <v>46314</v>
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Start/end dates are placeholders (not in the updates); confirm with the PO. EOC: subscription in Datadog, alerts at subscription level in progress. Help Desk T0 KBAs being revised. Help Desk asked to adopt ServiceNow or a Jira-ServiceNow integration; awaiting leadership. GovDelivery being considered instead of a DL for user notices. Source: COMET&lt;&gt;CMS PO updates.</t>
+          <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
       </c>
     </row>
@@ -2733,17 +2733,17 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Citrix to AVD user migration (6 waves)</t>
+          <t>AVD Feature Enhancements</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Expand hybrid &amp; multi-cloud hosting</t>
+          <t>Secure access &amp; compliance</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>Plan</t>
+          <t>Commit</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr">
@@ -2752,26 +2752,30 @@
         </is>
       </c>
       <c r="G30" s="15" t="n">
-        <v>46281</v>
+        <v>46259</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>46660</v>
+        <v>46568</v>
       </c>
       <c r="I30" s="13" t="n"/>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>Move Citrix users to AVD in six waves: validation and early adopters, then developers and RTI, then SAS and contractors.</t>
+          <t>Network, security and monitoring features (ZCC/Cloudflare, MFA, RTM, portal, host pools).</t>
         </is>
       </c>
       <c r="K30" s="13" t="n"/>
       <c r="L30" s="13" t="n"/>
-      <c r="M30" s="14" t="n"/>
+      <c r="M30" s="14" t="inlineStr">
+        <is>
+          <t>ZCC vs Cloudflare One decision blocked until the Cloudflare One POC is live. ECIS dependencies past their needed-by date: MFA setup (needed 8/25) and RTM permissions (needed 9/16). Network monitoring feasibility TBD.</t>
+        </is>
+      </c>
       <c r="N30" s="15" t="n">
-        <v>46302</v>
+        <v>46314</v>
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Dates are placeholders. Wave plan drafted and shared (9/23). Pilot interest: EOC team (9/23), AI Cohort team of 25 users (10/7, awaiting confirmation). Source: COMET&lt;&gt;CMS PO updates.</t>
+          <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
       </c>
     </row>
@@ -7089,12 +7093,10 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>AVD approved for an application ID in BaseCamp</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="n">
-        <v>46302</v>
-      </c>
+          <t>Patching - OS / System</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n"/>
       <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Release</t>
@@ -7102,7 +7104,7 @@
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F34" s="13" t="n"/>
@@ -7115,10 +7117,12 @@
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>Request AVD job code creation</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="n"/>
+          <t>Backup - Data Protect</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>46332</v>
+      </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Release</t>
@@ -7134,18 +7138,20 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>AVD-04</t>
+          <t>AVD-01</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>Decision: ServiceNow vs Jira-ServiceNow integration for support</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="n"/>
+          <t>Golden Image Management</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>46387</v>
+      </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
@@ -7158,18 +7164,20 @@
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>AVD-04</t>
+          <t>AVD-01</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>Decision: GovDelivery for user notifications</t>
-        </is>
-      </c>
-      <c r="C37" s="15" t="n"/>
+          <t>CrowdStrike Integration</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="n">
+        <v>46325</v>
+      </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -7182,25 +7190,25 @@
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>AVD-05</t>
+          <t>AVD-01</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Six-wave migration plan drafted and shared</t>
+          <t>Vulnerability Scanning</t>
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>46288</v>
+        <v>46660</v>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F38" s="13" t="n"/>
@@ -7208,18 +7216,20 @@
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>AVD-05</t>
+          <t>AVD-01</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Wave 0-2 pilot: EOC team and AI Cohort (25 users)</t>
-        </is>
-      </c>
-      <c r="C39" s="15" t="n"/>
+          <t>Autoscaling</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="n">
+        <v>46289</v>
+      </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -7232,17 +7242,15 @@
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>SCM-01</t>
+          <t>AVD-01</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Consolidated AWS TLS compliance dashboard (CloudFront + ELB)</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="n">
-        <v>46302</v>
-      </c>
+          <t>Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="n"/>
       <c r="D40" s="13" t="inlineStr">
         <is>
           <t>Release</t>
@@ -7250,7 +7258,7 @@
       </c>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F40" s="13" t="n"/>
@@ -7258,15 +7266,17 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>SCM-01</t>
+          <t>AVD-01</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>Azure and GCP TLS dashboards</t>
-        </is>
-      </c>
-      <c r="C41" s="15" t="n"/>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>46477</v>
+      </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
           <t>Release</t>
@@ -7282,16 +7292,16 @@
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>SCM-02</t>
+          <t>AVD-01</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>VPCConf export landing in Observability Hub S3 bucket</t>
+          <t>CCG Updates</t>
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>46302</v>
+        <v>46477</v>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
@@ -7300,7 +7310,7 @@
       </c>
       <c r="E42" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F42" s="13" t="n"/>
@@ -7308,15 +7318,17 @@
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>SCM-02</t>
+          <t>AVD-02</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>IP-to-account lookup table and app</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="n"/>
+          <t>AVD CLDSPT Requests</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>46318</v>
+      </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
           <t>Release</t>
@@ -7332,18 +7344,20 @@
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>SCM-03</t>
+          <t>AVD-02</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>CCG: Azure and GCP custom log collection approved by CMS</t>
-        </is>
-      </c>
-      <c r="C44" s="15" t="n"/>
+          <t>EOC Integration</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="n">
+        <v>46325</v>
+      </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -7356,25 +7370,25 @@
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>SCM-04</t>
+          <t>AVD-02</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>SplunkPS cost estimate delivered</t>
+          <t>CMS Help Desk</t>
         </is>
       </c>
       <c r="C45" s="15" t="n">
-        <v>46302</v>
+        <v>46353</v>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F45" s="13" t="n"/>
@@ -7382,16 +7396,16 @@
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>SCM-05</t>
+          <t>AVD-02</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>SDL starts GCP flow log ingestion</t>
+          <t>Distribution List / Gov Delivery</t>
         </is>
       </c>
       <c r="C46" s="15" t="n">
-        <v>46302</v>
+        <v>46360</v>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
@@ -7400,7 +7414,7 @@
       </c>
       <c r="E46" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F46" s="13" t="n"/>
@@ -7408,18 +7422,20 @@
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>SCM-05</t>
+          <t>AVD-02</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Funding decision: SDL instance in GCP</t>
-        </is>
-      </c>
-      <c r="C47" s="15" t="n"/>
+          <t>Cloud Tier 2</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="n">
+        <v>46477</v>
+      </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -7432,18 +7448,20 @@
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>SCM-07</t>
+          <t>AVD-02</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>MiSP plan for Cribl Search retrofit in AWS received</t>
-        </is>
-      </c>
-      <c r="C48" s="15" t="n"/>
+          <t>User Manual</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="n">
+        <v>46477</v>
+      </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
@@ -7456,16 +7474,16 @@
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>OBH-01</t>
+          <t>AVD-02</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>AD (Outpost) onboarded</t>
+          <t>Customer Support Team Training</t>
         </is>
       </c>
       <c r="C49" s="15" t="n">
-        <v>46281</v>
+        <v>46477</v>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
@@ -7474,7 +7492,7 @@
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F49" s="13" t="n"/>
@@ -7482,16 +7500,16 @@
     <row r="50">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>OBH-01</t>
+          <t>AVD-03</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>SMTP (Outpost) onboarded</t>
+          <t>Onboarding Process</t>
         </is>
       </c>
       <c r="C50" s="15" t="n">
-        <v>46288</v>
+        <v>46332</v>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
@@ -7500,7 +7518,7 @@
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F50" s="13" t="n"/>
@@ -7508,18 +7526,20 @@
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>OBH-01</t>
+          <t>AVD-04</t>
         </is>
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>6 MEF applications onboarded</t>
-        </is>
-      </c>
-      <c r="C51" s="15" t="n"/>
+          <t>Wave 0 - Validation only, no real users</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="n">
+        <v>46391</v>
+      </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Review gate</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -7532,15 +7552,17 @@
     <row r="52">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>OBH-03</t>
+          <t>AVD-04</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Azure ESS forwarding validated</t>
-        </is>
-      </c>
-      <c r="C52" s="15" t="n"/>
+          <t>Wave 1 - Admin Desktop (10)</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="n">
+        <v>46426</v>
+      </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
           <t>Release</t>
@@ -7556,15 +7578,17 @@
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>OBH-03</t>
+          <t>AVD-04</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>GCP ESS forwarding deployed to first account</t>
-        </is>
-      </c>
-      <c r="C53" s="15" t="n"/>
+          <t>Wave 2 - ECIS + Employees Desktop (60)</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="n">
+        <v>46454</v>
+      </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
           <t>Release</t>
@@ -7580,16 +7604,16 @@
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>OBH-04</t>
+          <t>AVD-04</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>BaseCAMP lookup tables created</t>
+          <t>Wave 3 - Developers Desktop (30, 8 vCPU/32GB)</t>
         </is>
       </c>
       <c r="C54" s="15" t="n">
-        <v>46288</v>
+        <v>46482</v>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
@@ -7598,7 +7622,7 @@
       </c>
       <c r="E54" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F54" s="13" t="n"/>
@@ -7606,15 +7630,17 @@
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>OBH-04</t>
+          <t>AVD-04</t>
         </is>
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>BaseCAMP lookup applied to EOC dashboard</t>
-        </is>
-      </c>
-      <c r="C55" s="15" t="n"/>
+          <t>Wave 4 - RTI Desktop (80)</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="n">
+        <v>46524</v>
+      </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
           <t>Release</t>
@@ -7630,217 +7656,629 @@
     <row r="56">
       <c r="A56" s="13" t="inlineStr">
         <is>
+          <t>AVD-04</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>Wave 5 - SAS PROD + Pre-Dev + VAL (260)</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="n">
+        <v>46566</v>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E56" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F56" s="13" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>AVD-04</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>Wave 6 - Contractors + Contractors 50G (605)</t>
+        </is>
+      </c>
+      <c r="C57" s="18" t="n">
+        <v>46594</v>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E57" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F57" s="16" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05</t>
+        </is>
+      </c>
+      <c r="B58" s="17" t="inlineStr">
+        <is>
+          <t>Zscaler Cloud Connector (ZCC) or Cloud Connector</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="n">
+        <v>46477</v>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>Real Time Monitoring</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="n">
+        <v>46303</v>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>MFA</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05</t>
+        </is>
+      </c>
+      <c r="B61" s="17" t="inlineStr">
+        <is>
+          <t>AVD Portal</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="n">
+        <v>46477</v>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05</t>
+        </is>
+      </c>
+      <c r="B62" s="17" t="inlineStr">
+        <is>
+          <t>Multi Session Host Pools</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="n">
+        <v>46568</v>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>Network Monitoring</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="n"/>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="inlineStr">
+        <is>
+          <t>SCM-01</t>
+        </is>
+      </c>
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>Consolidated AWS TLS compliance dashboard (CloudFront + ELB)</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="n">
+        <v>46302</v>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>SCM-01</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="inlineStr">
+        <is>
+          <t>Azure and GCP TLS dashboards</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="n"/>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F65" s="16" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="inlineStr">
+        <is>
+          <t>SCM-02</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>VPCConf export landing in Observability Hub S3 bucket</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="n">
+        <v>46302</v>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>SCM-02</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="inlineStr">
+        <is>
+          <t>IP-to-account lookup table and app</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="n"/>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="inlineStr">
+        <is>
+          <t>SCM-03</t>
+        </is>
+      </c>
+      <c r="B68" s="17" t="inlineStr">
+        <is>
+          <t>CCG: Azure and GCP custom log collection approved by CMS</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="n"/>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>SCM-04</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="inlineStr">
+        <is>
+          <t>SplunkPS cost estimate delivered</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="n">
+        <v>46302</v>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>SCM-05</t>
+        </is>
+      </c>
+      <c r="B70" s="17" t="inlineStr">
+        <is>
+          <t>SDL starts GCP flow log ingestion</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="n">
+        <v>46302</v>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F70" s="16" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>SCM-05</t>
+        </is>
+      </c>
+      <c r="B71" s="17" t="inlineStr">
+        <is>
+          <t>Funding decision: SDL instance in GCP</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="n"/>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t>SCM-07</t>
+        </is>
+      </c>
+      <c r="B72" s="17" t="inlineStr">
+        <is>
+          <t>MiSP plan for Cribl Search retrofit in AWS received</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="n"/>
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F72" s="16" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>OBH-01</t>
+        </is>
+      </c>
+      <c r="B73" s="17" t="inlineStr">
+        <is>
+          <t>AD (Outpost) onboarded</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
+          <t>OBH-01</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="inlineStr">
+        <is>
+          <t>SMTP (Outpost) onboarded</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="n">
+        <v>46288</v>
+      </c>
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F74" s="16" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>OBH-01</t>
+        </is>
+      </c>
+      <c r="B75" s="17" t="inlineStr">
+        <is>
+          <t>6 MEF applications onboarded</t>
+        </is>
+      </c>
+      <c r="C75" s="18" t="n"/>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>OBH-03</t>
+        </is>
+      </c>
+      <c r="B76" s="17" t="inlineStr">
+        <is>
+          <t>Azure ESS forwarding validated</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="n"/>
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F76" s="16" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="inlineStr">
+        <is>
+          <t>OBH-03</t>
+        </is>
+      </c>
+      <c r="B77" s="17" t="inlineStr">
+        <is>
+          <t>GCP ESS forwarding deployed to first account</t>
+        </is>
+      </c>
+      <c r="C77" s="18" t="n"/>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F77" s="16" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="16" t="inlineStr">
+        <is>
+          <t>OBH-04</t>
+        </is>
+      </c>
+      <c r="B78" s="17" t="inlineStr">
+        <is>
+          <t>BaseCAMP lookup tables created</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="n">
+        <v>46288</v>
+      </c>
+      <c r="D78" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F78" s="16" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>OBH-04</t>
+        </is>
+      </c>
+      <c r="B79" s="17" t="inlineStr">
+        <is>
+          <t>BaseCAMP lookup applied to EOC dashboard</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="n"/>
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F79" s="16" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
           <t>OBH-05</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B80" s="17" t="inlineStr">
         <is>
           <t>Cribl Replay demo</t>
         </is>
       </c>
-      <c r="C56" s="15" t="n"/>
-      <c r="D56" s="13" t="inlineStr">
+      <c r="C80" s="18" t="n"/>
+      <c r="D80" s="16" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="E56" s="13" t="inlineStr">
+      <c r="E80" s="16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F56" s="13" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="16" t="n"/>
-      <c r="B57" s="17" t="n"/>
-      <c r="C57" s="18" t="n"/>
-      <c r="D57" s="16" t="n"/>
-      <c r="E57" s="16" t="n"/>
-      <c r="F57" s="16" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="16" t="n"/>
-      <c r="B58" s="17" t="n"/>
-      <c r="C58" s="18" t="n"/>
-      <c r="D58" s="16" t="n"/>
-      <c r="E58" s="16" t="n"/>
-      <c r="F58" s="16" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="16" t="n"/>
-      <c r="B59" s="17" t="n"/>
-      <c r="C59" s="18" t="n"/>
-      <c r="D59" s="16" t="n"/>
-      <c r="E59" s="16" t="n"/>
-      <c r="F59" s="16" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="16" t="n"/>
-      <c r="B60" s="17" t="n"/>
-      <c r="C60" s="18" t="n"/>
-      <c r="D60" s="16" t="n"/>
-      <c r="E60" s="16" t="n"/>
-      <c r="F60" s="16" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="16" t="n"/>
-      <c r="B61" s="17" t="n"/>
-      <c r="C61" s="18" t="n"/>
-      <c r="D61" s="16" t="n"/>
-      <c r="E61" s="16" t="n"/>
-      <c r="F61" s="16" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="16" t="n"/>
-      <c r="B62" s="17" t="n"/>
-      <c r="C62" s="18" t="n"/>
-      <c r="D62" s="16" t="n"/>
-      <c r="E62" s="16" t="n"/>
-      <c r="F62" s="16" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="16" t="n"/>
-      <c r="B63" s="17" t="n"/>
-      <c r="C63" s="18" t="n"/>
-      <c r="D63" s="16" t="n"/>
-      <c r="E63" s="16" t="n"/>
-      <c r="F63" s="16" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="16" t="n"/>
-      <c r="B64" s="17" t="n"/>
-      <c r="C64" s="18" t="n"/>
-      <c r="D64" s="16" t="n"/>
-      <c r="E64" s="16" t="n"/>
-      <c r="F64" s="16" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="16" t="n"/>
-      <c r="B65" s="17" t="n"/>
-      <c r="C65" s="18" t="n"/>
-      <c r="D65" s="16" t="n"/>
-      <c r="E65" s="16" t="n"/>
-      <c r="F65" s="16" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="16" t="n"/>
-      <c r="B66" s="17" t="n"/>
-      <c r="C66" s="18" t="n"/>
-      <c r="D66" s="16" t="n"/>
-      <c r="E66" s="16" t="n"/>
-      <c r="F66" s="16" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="16" t="n"/>
-      <c r="B67" s="17" t="n"/>
-      <c r="C67" s="18" t="n"/>
-      <c r="D67" s="16" t="n"/>
-      <c r="E67" s="16" t="n"/>
-      <c r="F67" s="16" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="16" t="n"/>
-      <c r="B68" s="17" t="n"/>
-      <c r="C68" s="18" t="n"/>
-      <c r="D68" s="16" t="n"/>
-      <c r="E68" s="16" t="n"/>
-      <c r="F68" s="16" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="16" t="n"/>
-      <c r="B69" s="17" t="n"/>
-      <c r="C69" s="18" t="n"/>
-      <c r="D69" s="16" t="n"/>
-      <c r="E69" s="16" t="n"/>
-      <c r="F69" s="16" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="16" t="n"/>
-      <c r="B70" s="17" t="n"/>
-      <c r="C70" s="18" t="n"/>
-      <c r="D70" s="16" t="n"/>
-      <c r="E70" s="16" t="n"/>
-      <c r="F70" s="16" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="16" t="n"/>
-      <c r="B71" s="17" t="n"/>
-      <c r="C71" s="18" t="n"/>
-      <c r="D71" s="16" t="n"/>
-      <c r="E71" s="16" t="n"/>
-      <c r="F71" s="16" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="16" t="n"/>
-      <c r="B72" s="17" t="n"/>
-      <c r="C72" s="18" t="n"/>
-      <c r="D72" s="16" t="n"/>
-      <c r="E72" s="16" t="n"/>
-      <c r="F72" s="16" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="16" t="n"/>
-      <c r="B73" s="17" t="n"/>
-      <c r="C73" s="18" t="n"/>
-      <c r="D73" s="16" t="n"/>
-      <c r="E73" s="16" t="n"/>
-      <c r="F73" s="16" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="16" t="n"/>
-      <c r="B74" s="17" t="n"/>
-      <c r="C74" s="18" t="n"/>
-      <c r="D74" s="16" t="n"/>
-      <c r="E74" s="16" t="n"/>
-      <c r="F74" s="16" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="16" t="n"/>
-      <c r="B75" s="17" t="n"/>
-      <c r="C75" s="18" t="n"/>
-      <c r="D75" s="16" t="n"/>
-      <c r="E75" s="16" t="n"/>
-      <c r="F75" s="16" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="16" t="n"/>
-      <c r="B76" s="17" t="n"/>
-      <c r="C76" s="18" t="n"/>
-      <c r="D76" s="16" t="n"/>
-      <c r="E76" s="16" t="n"/>
-      <c r="F76" s="16" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="16" t="n"/>
-      <c r="B77" s="17" t="n"/>
-      <c r="C77" s="18" t="n"/>
-      <c r="D77" s="16" t="n"/>
-      <c r="E77" s="16" t="n"/>
-      <c r="F77" s="16" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="16" t="n"/>
-      <c r="B78" s="17" t="n"/>
-      <c r="C78" s="18" t="n"/>
-      <c r="D78" s="16" t="n"/>
-      <c r="E78" s="16" t="n"/>
-      <c r="F78" s="16" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="16" t="n"/>
-      <c r="B79" s="17" t="n"/>
-      <c r="C79" s="18" t="n"/>
-      <c r="D79" s="16" t="n"/>
-      <c r="E79" s="16" t="n"/>
-      <c r="F79" s="16" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="16" t="n"/>
-      <c r="B80" s="17" t="n"/>
-      <c r="C80" s="18" t="n"/>
-      <c r="D80" s="16" t="n"/>
-      <c r="E80" s="16" t="n"/>
       <c r="F80" s="16" t="n"/>
     </row>
     <row r="81">

</xml_diff>

<commit_message>
Show features under milestones; rename Initiative/Milestone to Milestone/Feature
</commit_message>
<xml_diff>
--- a/data/roadmaps/Roadmap - Combined.xlsx
+++ b/data/roadmaps/Roadmap - Combined.xlsx
@@ -6206,7 +6206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F201"/>
+  <dimension ref="A1:I201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6215,6 +6215,9 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6248,6 +6251,21 @@
           <t>Jira epic</t>
         </is>
       </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Start date</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Feature ID</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -6274,6 +6292,9 @@
         </is>
       </c>
       <c r="F2" s="13" t="n"/>
+      <c r="G2" s="15" t="n"/>
+      <c r="H2" s="13" t="n"/>
+      <c r="I2" s="13" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -6298,6 +6319,9 @@
         </is>
       </c>
       <c r="F3" s="13" t="n"/>
+      <c r="G3" s="15" t="n"/>
+      <c r="H3" s="13" t="n"/>
+      <c r="I3" s="13" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -6324,6 +6348,9 @@
         </is>
       </c>
       <c r="F4" s="13" t="n"/>
+      <c r="G4" s="15" t="n"/>
+      <c r="H4" s="13" t="n"/>
+      <c r="I4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -6350,6 +6377,9 @@
         </is>
       </c>
       <c r="F5" s="13" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="13" t="n"/>
+      <c r="I5" s="13" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -6374,6 +6404,9 @@
         </is>
       </c>
       <c r="F6" s="13" t="n"/>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="13" t="n"/>
+      <c r="I6" s="13" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -6398,6 +6431,9 @@
         </is>
       </c>
       <c r="F7" s="13" t="n"/>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="13" t="n"/>
+      <c r="I7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -6424,6 +6460,9 @@
         </is>
       </c>
       <c r="F8" s="13" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="13" t="n"/>
+      <c r="I8" s="13" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -6448,6 +6487,9 @@
         </is>
       </c>
       <c r="F9" s="13" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -6472,6 +6514,9 @@
         </is>
       </c>
       <c r="F10" s="13" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="13" t="n"/>
+      <c r="I10" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -6498,6 +6543,9 @@
         </is>
       </c>
       <c r="F11" s="13" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="13" t="n"/>
+      <c r="I11" s="13" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -6524,6 +6572,9 @@
         </is>
       </c>
       <c r="F12" s="13" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -6550,6 +6601,9 @@
         </is>
       </c>
       <c r="F13" s="13" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="13" t="n"/>
+      <c r="I13" s="13" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -6578,6 +6632,9 @@
           <t>CLDSPT-112641</t>
         </is>
       </c>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="13" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -6608,6 +6665,9 @@
           <t>CPT-6984</t>
         </is>
       </c>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="13" t="n"/>
+      <c r="I15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -6638,6 +6698,9 @@
           <t>CLDSPT-116097</t>
         </is>
       </c>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -6666,6 +6729,9 @@
           <t>CLDSPT-115656</t>
         </is>
       </c>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -6690,6 +6756,9 @@
         </is>
       </c>
       <c r="F18" s="13" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -6716,6 +6785,9 @@
         </is>
       </c>
       <c r="F19" s="13" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
@@ -6746,6 +6818,9 @@
           <t>FY26INIT-1097</t>
         </is>
       </c>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
@@ -6772,6 +6847,9 @@
         </is>
       </c>
       <c r="F21" s="13" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="13" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -6798,6 +6876,9 @@
         </is>
       </c>
       <c r="F22" s="13" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="13" t="n"/>
+      <c r="I22" s="13" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
@@ -6824,6 +6905,9 @@
         </is>
       </c>
       <c r="F23" s="13" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
@@ -6854,6 +6938,9 @@
           <t>CLDSPT-115520</t>
         </is>
       </c>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
@@ -6878,6 +6965,9 @@
         </is>
       </c>
       <c r="F25" s="13" t="n"/>
+      <c r="G25" s="15" t="n"/>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
@@ -6904,6 +6994,9 @@
         </is>
       </c>
       <c r="F26" s="13" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
@@ -6930,6 +7023,9 @@
         </is>
       </c>
       <c r="F27" s="13" t="n"/>
+      <c r="G27" s="15" t="n"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
@@ -6956,6 +7052,9 @@
         </is>
       </c>
       <c r="F28" s="13" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
@@ -6980,6 +7079,9 @@
         </is>
       </c>
       <c r="F29" s="13" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
@@ -7006,6 +7108,9 @@
         </is>
       </c>
       <c r="F30" s="13" t="n"/>
+      <c r="G30" s="15" t="n"/>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
@@ -7032,6 +7137,9 @@
         </is>
       </c>
       <c r="F31" s="13" t="n"/>
+      <c r="G31" s="15" t="n"/>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
@@ -7058,6 +7166,9 @@
         </is>
       </c>
       <c r="F32" s="13" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
@@ -7084,6 +7195,9 @@
         </is>
       </c>
       <c r="F33" s="13" t="n"/>
+      <c r="G33" s="15" t="n"/>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="13" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
@@ -7108,6 +7222,17 @@
         </is>
       </c>
       <c r="F34" s="13" t="n"/>
+      <c r="G34" s="15" t="n"/>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.1</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>MiSP</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
@@ -7134,6 +7259,19 @@
         </is>
       </c>
       <c r="F35" s="13" t="n"/>
+      <c r="G35" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.2</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>IaaS</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
@@ -7160,6 +7298,19 @@
         </is>
       </c>
       <c r="F36" s="13" t="n"/>
+      <c r="G36" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.3</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>SecOps</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
@@ -7186,6 +7337,19 @@
         </is>
       </c>
       <c r="F37" s="13" t="n"/>
+      <c r="G37" s="15" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.4</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>SecOps</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
@@ -7212,6 +7376,19 @@
         </is>
       </c>
       <c r="F38" s="13" t="n"/>
+      <c r="G38" s="15" t="n">
+        <v>46569</v>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.9</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>COMET / SecOps</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
@@ -7238,6 +7415,19 @@
         </is>
       </c>
       <c r="F39" s="13" t="n"/>
+      <c r="G39" s="15" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.5</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
@@ -7262,6 +7452,17 @@
         </is>
       </c>
       <c r="F40" s="13" t="n"/>
+      <c r="G40" s="15" t="n"/>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.6</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>IaaS / COMET</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
@@ -7288,6 +7489,19 @@
         </is>
       </c>
       <c r="F41" s="13" t="n"/>
+      <c r="G41" s="15" t="n">
+        <v>46388</v>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.7</t>
+        </is>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
@@ -7314,6 +7528,19 @@
         </is>
       </c>
       <c r="F42" s="13" t="n"/>
+      <c r="G42" s="15" t="n">
+        <v>46388</v>
+      </c>
+      <c r="H42" s="13" t="inlineStr">
+        <is>
+          <t>AVD-01.8</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>COMET / CSS</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
@@ -7340,6 +7567,19 @@
         </is>
       </c>
       <c r="F43" s="13" t="n"/>
+      <c r="G43" s="15" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H43" s="13" t="inlineStr">
+        <is>
+          <t>AVD-02.1</t>
+        </is>
+      </c>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>COMET (Atlassian)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
@@ -7366,6 +7606,19 @@
         </is>
       </c>
       <c r="F44" s="13" t="n"/>
+      <c r="G44" s="15" t="n">
+        <v>46262</v>
+      </c>
+      <c r="H44" s="13" t="inlineStr">
+        <is>
+          <t>AVD-02.2</t>
+        </is>
+      </c>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>SRE Team</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
@@ -7392,6 +7645,19 @@
         </is>
       </c>
       <c r="F45" s="13" t="n"/>
+      <c r="G45" s="15" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H45" s="13" t="inlineStr">
+        <is>
+          <t>AVD-02.3</t>
+        </is>
+      </c>
+      <c r="I45" s="13" t="inlineStr">
+        <is>
+          <t>CMS Help Desk / Nerdio CSM</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
@@ -7418,6 +7684,19 @@
         </is>
       </c>
       <c r="F46" s="13" t="n"/>
+      <c r="G46" s="15" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H46" s="13" t="inlineStr">
+        <is>
+          <t>AVD-02.4</t>
+        </is>
+      </c>
+      <c r="I46" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
@@ -7444,6 +7723,19 @@
         </is>
       </c>
       <c r="F47" s="13" t="n"/>
+      <c r="G47" s="15" t="n">
+        <v>46388</v>
+      </c>
+      <c r="H47" s="13" t="inlineStr">
+        <is>
+          <t>AVD-02.5</t>
+        </is>
+      </c>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
@@ -7470,6 +7762,19 @@
         </is>
       </c>
       <c r="F48" s="13" t="n"/>
+      <c r="G48" s="15" t="n">
+        <v>46388</v>
+      </c>
+      <c r="H48" s="13" t="inlineStr">
+        <is>
+          <t>AVD-02.6</t>
+        </is>
+      </c>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
@@ -7496,6 +7801,19 @@
         </is>
       </c>
       <c r="F49" s="13" t="n"/>
+      <c r="G49" s="15" t="n">
+        <v>46388</v>
+      </c>
+      <c r="H49" s="13" t="inlineStr">
+        <is>
+          <t>AVD-02.7</t>
+        </is>
+      </c>
+      <c r="I49" s="13" t="inlineStr">
+        <is>
+          <t>COMET / CSS</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="13" t="inlineStr">
@@ -7522,6 +7840,19 @@
         </is>
       </c>
       <c r="F50" s="13" t="n"/>
+      <c r="G50" s="15" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>AVD-03.1</t>
+        </is>
+      </c>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
@@ -7548,6 +7879,19 @@
         </is>
       </c>
       <c r="F51" s="13" t="n"/>
+      <c r="G51" s="15" t="n">
+        <v>46391</v>
+      </c>
+      <c r="H51" s="13" t="inlineStr">
+        <is>
+          <t>AVD-04.1</t>
+        </is>
+      </c>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="13" t="inlineStr">
@@ -7574,6 +7918,19 @@
         </is>
       </c>
       <c r="F52" s="13" t="n"/>
+      <c r="G52" s="15" t="n">
+        <v>46426</v>
+      </c>
+      <c r="H52" s="13" t="inlineStr">
+        <is>
+          <t>AVD-04.2</t>
+        </is>
+      </c>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
@@ -7600,6 +7957,19 @@
         </is>
       </c>
       <c r="F53" s="13" t="n"/>
+      <c r="G53" s="15" t="n">
+        <v>46454</v>
+      </c>
+      <c r="H53" s="13" t="inlineStr">
+        <is>
+          <t>AVD-04.3</t>
+        </is>
+      </c>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
@@ -7626,6 +7996,19 @@
         </is>
       </c>
       <c r="F54" s="13" t="n"/>
+      <c r="G54" s="15" t="n">
+        <v>46482</v>
+      </c>
+      <c r="H54" s="13" t="inlineStr">
+        <is>
+          <t>AVD-04.4</t>
+        </is>
+      </c>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
@@ -7652,6 +8035,19 @@
         </is>
       </c>
       <c r="F55" s="13" t="n"/>
+      <c r="G55" s="15" t="n">
+        <v>46524</v>
+      </c>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>AVD-04.5</t>
+        </is>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="13" t="inlineStr">
@@ -7678,6 +8074,19 @@
         </is>
       </c>
       <c r="F56" s="13" t="n"/>
+      <c r="G56" s="15" t="n">
+        <v>46566</v>
+      </c>
+      <c r="H56" s="13" t="inlineStr">
+        <is>
+          <t>AVD-04.6</t>
+        </is>
+      </c>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
@@ -7704,6 +8113,19 @@
         </is>
       </c>
       <c r="F57" s="16" t="n"/>
+      <c r="G57" s="18" t="n">
+        <v>46594</v>
+      </c>
+      <c r="H57" s="16" t="inlineStr">
+        <is>
+          <t>AVD-04.7</t>
+        </is>
+      </c>
+      <c r="I57" s="16" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
@@ -7730,6 +8152,19 @@
         </is>
       </c>
       <c r="F58" s="16" t="n"/>
+      <c r="G58" s="18" t="n">
+        <v>46388</v>
+      </c>
+      <c r="H58" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05.1</t>
+        </is>
+      </c>
+      <c r="I58" s="16" t="inlineStr">
+        <is>
+          <t>NetOps</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
@@ -7756,6 +8191,19 @@
         </is>
       </c>
       <c r="F59" s="16" t="n"/>
+      <c r="G59" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H59" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05.2</t>
+        </is>
+      </c>
+      <c r="I59" s="16" t="inlineStr">
+        <is>
+          <t>ECIS</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
@@ -7782,6 +8230,19 @@
         </is>
       </c>
       <c r="F60" s="16" t="n"/>
+      <c r="G60" s="18" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H60" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05.3</t>
+        </is>
+      </c>
+      <c r="I60" s="16" t="inlineStr">
+        <is>
+          <t>ECIS</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
@@ -7808,6 +8269,19 @@
         </is>
       </c>
       <c r="F61" s="16" t="n"/>
+      <c r="G61" s="18" t="n">
+        <v>46388</v>
+      </c>
+      <c r="H61" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05.4</t>
+        </is>
+      </c>
+      <c r="I61" s="16" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
@@ -7834,6 +8308,19 @@
         </is>
       </c>
       <c r="F62" s="16" t="n"/>
+      <c r="G62" s="18" t="n">
+        <v>46478</v>
+      </c>
+      <c r="H62" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05.5</t>
+        </is>
+      </c>
+      <c r="I62" s="16" t="inlineStr">
+        <is>
+          <t>COMET</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="16" t="inlineStr">
@@ -7858,6 +8345,17 @@
         </is>
       </c>
       <c r="F63" s="16" t="n"/>
+      <c r="G63" s="18" t="n"/>
+      <c r="H63" s="16" t="inlineStr">
+        <is>
+          <t>AVD-05.6</t>
+        </is>
+      </c>
+      <c r="I63" s="16" t="inlineStr">
+        <is>
+          <t>NetOps</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
@@ -7884,6 +8382,9 @@
         </is>
       </c>
       <c r="F64" s="16" t="n"/>
+      <c r="G64" s="18" t="n"/>
+      <c r="H64" s="16" t="n"/>
+      <c r="I64" s="16" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
@@ -7908,6 +8409,9 @@
         </is>
       </c>
       <c r="F65" s="16" t="n"/>
+      <c r="G65" s="18" t="n"/>
+      <c r="H65" s="16" t="n"/>
+      <c r="I65" s="16" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="16" t="inlineStr">
@@ -7934,6 +8438,9 @@
         </is>
       </c>
       <c r="F66" s="16" t="n"/>
+      <c r="G66" s="18" t="n"/>
+      <c r="H66" s="16" t="n"/>
+      <c r="I66" s="16" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
@@ -7958,6 +8465,9 @@
         </is>
       </c>
       <c r="F67" s="16" t="n"/>
+      <c r="G67" s="18" t="n"/>
+      <c r="H67" s="16" t="n"/>
+      <c r="I67" s="16" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
@@ -7982,6 +8492,9 @@
         </is>
       </c>
       <c r="F68" s="16" t="n"/>
+      <c r="G68" s="18" t="n"/>
+      <c r="H68" s="16" t="n"/>
+      <c r="I68" s="16" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -8008,6 +8521,9 @@
         </is>
       </c>
       <c r="F69" s="16" t="n"/>
+      <c r="G69" s="18" t="n"/>
+      <c r="H69" s="16" t="n"/>
+      <c r="I69" s="16" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="16" t="inlineStr">
@@ -8034,6 +8550,9 @@
         </is>
       </c>
       <c r="F70" s="16" t="n"/>
+      <c r="G70" s="18" t="n"/>
+      <c r="H70" s="16" t="n"/>
+      <c r="I70" s="16" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="16" t="inlineStr">
@@ -8058,6 +8577,9 @@
         </is>
       </c>
       <c r="F71" s="16" t="n"/>
+      <c r="G71" s="18" t="n"/>
+      <c r="H71" s="16" t="n"/>
+      <c r="I71" s="16" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
@@ -8082,6 +8604,9 @@
         </is>
       </c>
       <c r="F72" s="16" t="n"/>
+      <c r="G72" s="18" t="n"/>
+      <c r="H72" s="16" t="n"/>
+      <c r="I72" s="16" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
@@ -8108,6 +8633,9 @@
         </is>
       </c>
       <c r="F73" s="16" t="n"/>
+      <c r="G73" s="18" t="n"/>
+      <c r="H73" s="16" t="n"/>
+      <c r="I73" s="16" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
@@ -8134,6 +8662,9 @@
         </is>
       </c>
       <c r="F74" s="16" t="n"/>
+      <c r="G74" s="18" t="n"/>
+      <c r="H74" s="16" t="n"/>
+      <c r="I74" s="16" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="16" t="inlineStr">
@@ -8158,6 +8689,9 @@
         </is>
       </c>
       <c r="F75" s="16" t="n"/>
+      <c r="G75" s="18" t="n"/>
+      <c r="H75" s="16" t="n"/>
+      <c r="I75" s="16" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="16" t="inlineStr">
@@ -8182,6 +8716,9 @@
         </is>
       </c>
       <c r="F76" s="16" t="n"/>
+      <c r="G76" s="18" t="n"/>
+      <c r="H76" s="16" t="n"/>
+      <c r="I76" s="16" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
@@ -8206,6 +8743,9 @@
         </is>
       </c>
       <c r="F77" s="16" t="n"/>
+      <c r="G77" s="18" t="n"/>
+      <c r="H77" s="16" t="n"/>
+      <c r="I77" s="16" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="16" t="inlineStr">
@@ -8232,6 +8772,9 @@
         </is>
       </c>
       <c r="F78" s="16" t="n"/>
+      <c r="G78" s="18" t="n"/>
+      <c r="H78" s="16" t="n"/>
+      <c r="I78" s="16" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="16" t="inlineStr">
@@ -8256,6 +8799,9 @@
         </is>
       </c>
       <c r="F79" s="16" t="n"/>
+      <c r="G79" s="18" t="n"/>
+      <c r="H79" s="16" t="n"/>
+      <c r="I79" s="16" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
@@ -8280,6 +8826,9 @@
         </is>
       </c>
       <c r="F80" s="16" t="n"/>
+      <c r="G80" s="18" t="n"/>
+      <c r="H80" s="16" t="n"/>
+      <c r="I80" s="16" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="16" t="n"/>
@@ -8288,6 +8837,9 @@
       <c r="D81" s="16" t="n"/>
       <c r="E81" s="16" t="n"/>
       <c r="F81" s="16" t="n"/>
+      <c r="G81" s="18" t="n"/>
+      <c r="H81" s="16" t="n"/>
+      <c r="I81" s="16" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="16" t="n"/>
@@ -8296,6 +8848,9 @@
       <c r="D82" s="16" t="n"/>
       <c r="E82" s="16" t="n"/>
       <c r="F82" s="16" t="n"/>
+      <c r="G82" s="18" t="n"/>
+      <c r="H82" s="16" t="n"/>
+      <c r="I82" s="16" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="16" t="n"/>
@@ -8304,6 +8859,9 @@
       <c r="D83" s="16" t="n"/>
       <c r="E83" s="16" t="n"/>
       <c r="F83" s="16" t="n"/>
+      <c r="G83" s="18" t="n"/>
+      <c r="H83" s="16" t="n"/>
+      <c r="I83" s="16" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="16" t="n"/>
@@ -8312,6 +8870,9 @@
       <c r="D84" s="16" t="n"/>
       <c r="E84" s="16" t="n"/>
       <c r="F84" s="16" t="n"/>
+      <c r="G84" s="18" t="n"/>
+      <c r="H84" s="16" t="n"/>
+      <c r="I84" s="16" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="16" t="n"/>
@@ -8320,6 +8881,9 @@
       <c r="D85" s="16" t="n"/>
       <c r="E85" s="16" t="n"/>
       <c r="F85" s="16" t="n"/>
+      <c r="G85" s="18" t="n"/>
+      <c r="H85" s="16" t="n"/>
+      <c r="I85" s="16" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="16" t="n"/>
@@ -8328,6 +8892,9 @@
       <c r="D86" s="16" t="n"/>
       <c r="E86" s="16" t="n"/>
       <c r="F86" s="16" t="n"/>
+      <c r="G86" s="18" t="n"/>
+      <c r="H86" s="16" t="n"/>
+      <c r="I86" s="16" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="16" t="n"/>
@@ -8336,6 +8903,9 @@
       <c r="D87" s="16" t="n"/>
       <c r="E87" s="16" t="n"/>
       <c r="F87" s="16" t="n"/>
+      <c r="G87" s="18" t="n"/>
+      <c r="H87" s="16" t="n"/>
+      <c r="I87" s="16" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="16" t="n"/>
@@ -8344,6 +8914,9 @@
       <c r="D88" s="16" t="n"/>
       <c r="E88" s="16" t="n"/>
       <c r="F88" s="16" t="n"/>
+      <c r="G88" s="18" t="n"/>
+      <c r="H88" s="16" t="n"/>
+      <c r="I88" s="16" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="16" t="n"/>
@@ -8352,6 +8925,9 @@
       <c r="D89" s="16" t="n"/>
       <c r="E89" s="16" t="n"/>
       <c r="F89" s="16" t="n"/>
+      <c r="G89" s="18" t="n"/>
+      <c r="H89" s="16" t="n"/>
+      <c r="I89" s="16" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="16" t="n"/>
@@ -8360,6 +8936,9 @@
       <c r="D90" s="16" t="n"/>
       <c r="E90" s="16" t="n"/>
       <c r="F90" s="16" t="n"/>
+      <c r="G90" s="18" t="n"/>
+      <c r="H90" s="16" t="n"/>
+      <c r="I90" s="16" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="16" t="n"/>
@@ -8368,6 +8947,9 @@
       <c r="D91" s="16" t="n"/>
       <c r="E91" s="16" t="n"/>
       <c r="F91" s="16" t="n"/>
+      <c r="G91" s="18" t="n"/>
+      <c r="H91" s="16" t="n"/>
+      <c r="I91" s="16" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="16" t="n"/>
@@ -8376,6 +8958,9 @@
       <c r="D92" s="16" t="n"/>
       <c r="E92" s="16" t="n"/>
       <c r="F92" s="16" t="n"/>
+      <c r="G92" s="18" t="n"/>
+      <c r="H92" s="16" t="n"/>
+      <c r="I92" s="16" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="16" t="n"/>
@@ -8384,6 +8969,9 @@
       <c r="D93" s="16" t="n"/>
       <c r="E93" s="16" t="n"/>
       <c r="F93" s="16" t="n"/>
+      <c r="G93" s="18" t="n"/>
+      <c r="H93" s="16" t="n"/>
+      <c r="I93" s="16" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="16" t="n"/>
@@ -8392,6 +8980,9 @@
       <c r="D94" s="16" t="n"/>
       <c r="E94" s="16" t="n"/>
       <c r="F94" s="16" t="n"/>
+      <c r="G94" s="18" t="n"/>
+      <c r="H94" s="16" t="n"/>
+      <c r="I94" s="16" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="16" t="n"/>
@@ -8400,6 +8991,9 @@
       <c r="D95" s="16" t="n"/>
       <c r="E95" s="16" t="n"/>
       <c r="F95" s="16" t="n"/>
+      <c r="G95" s="18" t="n"/>
+      <c r="H95" s="16" t="n"/>
+      <c r="I95" s="16" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="16" t="n"/>
@@ -8408,6 +9002,9 @@
       <c r="D96" s="16" t="n"/>
       <c r="E96" s="16" t="n"/>
       <c r="F96" s="16" t="n"/>
+      <c r="G96" s="18" t="n"/>
+      <c r="H96" s="16" t="n"/>
+      <c r="I96" s="16" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="16" t="n"/>
@@ -8416,6 +9013,9 @@
       <c r="D97" s="16" t="n"/>
       <c r="E97" s="16" t="n"/>
       <c r="F97" s="16" t="n"/>
+      <c r="G97" s="18" t="n"/>
+      <c r="H97" s="16" t="n"/>
+      <c r="I97" s="16" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="16" t="n"/>
@@ -8424,6 +9024,9 @@
       <c r="D98" s="16" t="n"/>
       <c r="E98" s="16" t="n"/>
       <c r="F98" s="16" t="n"/>
+      <c r="G98" s="18" t="n"/>
+      <c r="H98" s="16" t="n"/>
+      <c r="I98" s="16" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="16" t="n"/>
@@ -8432,6 +9035,9 @@
       <c r="D99" s="16" t="n"/>
       <c r="E99" s="16" t="n"/>
       <c r="F99" s="16" t="n"/>
+      <c r="G99" s="18" t="n"/>
+      <c r="H99" s="16" t="n"/>
+      <c r="I99" s="16" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="16" t="n"/>
@@ -8440,6 +9046,9 @@
       <c r="D100" s="16" t="n"/>
       <c r="E100" s="16" t="n"/>
       <c r="F100" s="16" t="n"/>
+      <c r="G100" s="18" t="n"/>
+      <c r="H100" s="16" t="n"/>
+      <c r="I100" s="16" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="16" t="n"/>
@@ -8448,6 +9057,9 @@
       <c r="D101" s="16" t="n"/>
       <c r="E101" s="16" t="n"/>
       <c r="F101" s="16" t="n"/>
+      <c r="G101" s="18" t="n"/>
+      <c r="H101" s="16" t="n"/>
+      <c r="I101" s="16" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="16" t="n"/>
@@ -8456,6 +9068,9 @@
       <c r="D102" s="16" t="n"/>
       <c r="E102" s="16" t="n"/>
       <c r="F102" s="16" t="n"/>
+      <c r="G102" s="18" t="n"/>
+      <c r="H102" s="16" t="n"/>
+      <c r="I102" s="16" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="16" t="n"/>
@@ -8464,6 +9079,9 @@
       <c r="D103" s="16" t="n"/>
       <c r="E103" s="16" t="n"/>
       <c r="F103" s="16" t="n"/>
+      <c r="G103" s="18" t="n"/>
+      <c r="H103" s="16" t="n"/>
+      <c r="I103" s="16" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="16" t="n"/>
@@ -8472,6 +9090,9 @@
       <c r="D104" s="16" t="n"/>
       <c r="E104" s="16" t="n"/>
       <c r="F104" s="16" t="n"/>
+      <c r="G104" s="18" t="n"/>
+      <c r="H104" s="16" t="n"/>
+      <c r="I104" s="16" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="16" t="n"/>
@@ -8480,6 +9101,9 @@
       <c r="D105" s="16" t="n"/>
       <c r="E105" s="16" t="n"/>
       <c r="F105" s="16" t="n"/>
+      <c r="G105" s="18" t="n"/>
+      <c r="H105" s="16" t="n"/>
+      <c r="I105" s="16" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="16" t="n"/>
@@ -8488,6 +9112,9 @@
       <c r="D106" s="16" t="n"/>
       <c r="E106" s="16" t="n"/>
       <c r="F106" s="16" t="n"/>
+      <c r="G106" s="18" t="n"/>
+      <c r="H106" s="16" t="n"/>
+      <c r="I106" s="16" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="16" t="n"/>
@@ -8496,6 +9123,9 @@
       <c r="D107" s="16" t="n"/>
       <c r="E107" s="16" t="n"/>
       <c r="F107" s="16" t="n"/>
+      <c r="G107" s="18" t="n"/>
+      <c r="H107" s="16" t="n"/>
+      <c r="I107" s="16" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="16" t="n"/>
@@ -8504,6 +9134,9 @@
       <c r="D108" s="16" t="n"/>
       <c r="E108" s="16" t="n"/>
       <c r="F108" s="16" t="n"/>
+      <c r="G108" s="18" t="n"/>
+      <c r="H108" s="16" t="n"/>
+      <c r="I108" s="16" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="16" t="n"/>
@@ -8512,6 +9145,9 @@
       <c r="D109" s="16" t="n"/>
       <c r="E109" s="16" t="n"/>
       <c r="F109" s="16" t="n"/>
+      <c r="G109" s="18" t="n"/>
+      <c r="H109" s="16" t="n"/>
+      <c r="I109" s="16" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="16" t="n"/>
@@ -8520,6 +9156,9 @@
       <c r="D110" s="16" t="n"/>
       <c r="E110" s="16" t="n"/>
       <c r="F110" s="16" t="n"/>
+      <c r="G110" s="18" t="n"/>
+      <c r="H110" s="16" t="n"/>
+      <c r="I110" s="16" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="16" t="n"/>
@@ -8528,6 +9167,9 @@
       <c r="D111" s="16" t="n"/>
       <c r="E111" s="16" t="n"/>
       <c r="F111" s="16" t="n"/>
+      <c r="G111" s="18" t="n"/>
+      <c r="H111" s="16" t="n"/>
+      <c r="I111" s="16" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="16" t="n"/>
@@ -8536,6 +9178,9 @@
       <c r="D112" s="16" t="n"/>
       <c r="E112" s="16" t="n"/>
       <c r="F112" s="16" t="n"/>
+      <c r="G112" s="18" t="n"/>
+      <c r="H112" s="16" t="n"/>
+      <c r="I112" s="16" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="16" t="n"/>
@@ -8544,6 +9189,9 @@
       <c r="D113" s="16" t="n"/>
       <c r="E113" s="16" t="n"/>
       <c r="F113" s="16" t="n"/>
+      <c r="G113" s="18" t="n"/>
+      <c r="H113" s="16" t="n"/>
+      <c r="I113" s="16" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="16" t="n"/>
@@ -8552,6 +9200,9 @@
       <c r="D114" s="16" t="n"/>
       <c r="E114" s="16" t="n"/>
       <c r="F114" s="16" t="n"/>
+      <c r="G114" s="18" t="n"/>
+      <c r="H114" s="16" t="n"/>
+      <c r="I114" s="16" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="16" t="n"/>
@@ -8560,6 +9211,9 @@
       <c r="D115" s="16" t="n"/>
       <c r="E115" s="16" t="n"/>
       <c r="F115" s="16" t="n"/>
+      <c r="G115" s="18" t="n"/>
+      <c r="H115" s="16" t="n"/>
+      <c r="I115" s="16" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="16" t="n"/>
@@ -8568,6 +9222,9 @@
       <c r="D116" s="16" t="n"/>
       <c r="E116" s="16" t="n"/>
       <c r="F116" s="16" t="n"/>
+      <c r="G116" s="18" t="n"/>
+      <c r="H116" s="16" t="n"/>
+      <c r="I116" s="16" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="16" t="n"/>
@@ -8576,6 +9233,9 @@
       <c r="D117" s="16" t="n"/>
       <c r="E117" s="16" t="n"/>
       <c r="F117" s="16" t="n"/>
+      <c r="G117" s="18" t="n"/>
+      <c r="H117" s="16" t="n"/>
+      <c r="I117" s="16" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="16" t="n"/>
@@ -8584,6 +9244,9 @@
       <c r="D118" s="16" t="n"/>
       <c r="E118" s="16" t="n"/>
       <c r="F118" s="16" t="n"/>
+      <c r="G118" s="18" t="n"/>
+      <c r="H118" s="16" t="n"/>
+      <c r="I118" s="16" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="16" t="n"/>
@@ -8592,6 +9255,9 @@
       <c r="D119" s="16" t="n"/>
       <c r="E119" s="16" t="n"/>
       <c r="F119" s="16" t="n"/>
+      <c r="G119" s="18" t="n"/>
+      <c r="H119" s="16" t="n"/>
+      <c r="I119" s="16" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="16" t="n"/>
@@ -8600,6 +9266,9 @@
       <c r="D120" s="16" t="n"/>
       <c r="E120" s="16" t="n"/>
       <c r="F120" s="16" t="n"/>
+      <c r="G120" s="18" t="n"/>
+      <c r="H120" s="16" t="n"/>
+      <c r="I120" s="16" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="16" t="n"/>
@@ -8608,6 +9277,9 @@
       <c r="D121" s="16" t="n"/>
       <c r="E121" s="16" t="n"/>
       <c r="F121" s="16" t="n"/>
+      <c r="G121" s="18" t="n"/>
+      <c r="H121" s="16" t="n"/>
+      <c r="I121" s="16" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="16" t="n"/>
@@ -8616,6 +9288,9 @@
       <c r="D122" s="16" t="n"/>
       <c r="E122" s="16" t="n"/>
       <c r="F122" s="16" t="n"/>
+      <c r="G122" s="18" t="n"/>
+      <c r="H122" s="16" t="n"/>
+      <c r="I122" s="16" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="16" t="n"/>
@@ -8624,6 +9299,9 @@
       <c r="D123" s="16" t="n"/>
       <c r="E123" s="16" t="n"/>
       <c r="F123" s="16" t="n"/>
+      <c r="G123" s="18" t="n"/>
+      <c r="H123" s="16" t="n"/>
+      <c r="I123" s="16" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="16" t="n"/>
@@ -8632,6 +9310,9 @@
       <c r="D124" s="16" t="n"/>
       <c r="E124" s="16" t="n"/>
       <c r="F124" s="16" t="n"/>
+      <c r="G124" s="18" t="n"/>
+      <c r="H124" s="16" t="n"/>
+      <c r="I124" s="16" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="16" t="n"/>
@@ -8640,6 +9321,9 @@
       <c r="D125" s="16" t="n"/>
       <c r="E125" s="16" t="n"/>
       <c r="F125" s="16" t="n"/>
+      <c r="G125" s="18" t="n"/>
+      <c r="H125" s="16" t="n"/>
+      <c r="I125" s="16" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="16" t="n"/>
@@ -8648,6 +9332,9 @@
       <c r="D126" s="16" t="n"/>
       <c r="E126" s="16" t="n"/>
       <c r="F126" s="16" t="n"/>
+      <c r="G126" s="18" t="n"/>
+      <c r="H126" s="16" t="n"/>
+      <c r="I126" s="16" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="16" t="n"/>
@@ -8656,6 +9343,9 @@
       <c r="D127" s="16" t="n"/>
       <c r="E127" s="16" t="n"/>
       <c r="F127" s="16" t="n"/>
+      <c r="G127" s="18" t="n"/>
+      <c r="H127" s="16" t="n"/>
+      <c r="I127" s="16" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="16" t="n"/>
@@ -8664,6 +9354,9 @@
       <c r="D128" s="16" t="n"/>
       <c r="E128" s="16" t="n"/>
       <c r="F128" s="16" t="n"/>
+      <c r="G128" s="18" t="n"/>
+      <c r="H128" s="16" t="n"/>
+      <c r="I128" s="16" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="16" t="n"/>
@@ -8672,6 +9365,9 @@
       <c r="D129" s="16" t="n"/>
       <c r="E129" s="16" t="n"/>
       <c r="F129" s="16" t="n"/>
+      <c r="G129" s="18" t="n"/>
+      <c r="H129" s="16" t="n"/>
+      <c r="I129" s="16" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="16" t="n"/>
@@ -8680,6 +9376,9 @@
       <c r="D130" s="16" t="n"/>
       <c r="E130" s="16" t="n"/>
       <c r="F130" s="16" t="n"/>
+      <c r="G130" s="18" t="n"/>
+      <c r="H130" s="16" t="n"/>
+      <c r="I130" s="16" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="16" t="n"/>
@@ -8688,6 +9387,9 @@
       <c r="D131" s="16" t="n"/>
       <c r="E131" s="16" t="n"/>
       <c r="F131" s="16" t="n"/>
+      <c r="G131" s="18" t="n"/>
+      <c r="H131" s="16" t="n"/>
+      <c r="I131" s="16" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="16" t="n"/>
@@ -8696,6 +9398,9 @@
       <c r="D132" s="16" t="n"/>
       <c r="E132" s="16" t="n"/>
       <c r="F132" s="16" t="n"/>
+      <c r="G132" s="18" t="n"/>
+      <c r="H132" s="16" t="n"/>
+      <c r="I132" s="16" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="16" t="n"/>
@@ -8704,6 +9409,9 @@
       <c r="D133" s="16" t="n"/>
       <c r="E133" s="16" t="n"/>
       <c r="F133" s="16" t="n"/>
+      <c r="G133" s="18" t="n"/>
+      <c r="H133" s="16" t="n"/>
+      <c r="I133" s="16" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="16" t="n"/>
@@ -8712,6 +9420,9 @@
       <c r="D134" s="16" t="n"/>
       <c r="E134" s="16" t="n"/>
       <c r="F134" s="16" t="n"/>
+      <c r="G134" s="18" t="n"/>
+      <c r="H134" s="16" t="n"/>
+      <c r="I134" s="16" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="16" t="n"/>
@@ -8720,6 +9431,9 @@
       <c r="D135" s="16" t="n"/>
       <c r="E135" s="16" t="n"/>
       <c r="F135" s="16" t="n"/>
+      <c r="G135" s="18" t="n"/>
+      <c r="H135" s="16" t="n"/>
+      <c r="I135" s="16" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="16" t="n"/>
@@ -8728,6 +9442,9 @@
       <c r="D136" s="16" t="n"/>
       <c r="E136" s="16" t="n"/>
       <c r="F136" s="16" t="n"/>
+      <c r="G136" s="18" t="n"/>
+      <c r="H136" s="16" t="n"/>
+      <c r="I136" s="16" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="16" t="n"/>
@@ -8736,6 +9453,9 @@
       <c r="D137" s="16" t="n"/>
       <c r="E137" s="16" t="n"/>
       <c r="F137" s="16" t="n"/>
+      <c r="G137" s="18" t="n"/>
+      <c r="H137" s="16" t="n"/>
+      <c r="I137" s="16" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="16" t="n"/>
@@ -8744,6 +9464,9 @@
       <c r="D138" s="16" t="n"/>
       <c r="E138" s="16" t="n"/>
       <c r="F138" s="16" t="n"/>
+      <c r="G138" s="18" t="n"/>
+      <c r="H138" s="16" t="n"/>
+      <c r="I138" s="16" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="16" t="n"/>
@@ -8752,6 +9475,9 @@
       <c r="D139" s="16" t="n"/>
       <c r="E139" s="16" t="n"/>
       <c r="F139" s="16" t="n"/>
+      <c r="G139" s="18" t="n"/>
+      <c r="H139" s="16" t="n"/>
+      <c r="I139" s="16" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="16" t="n"/>
@@ -8760,6 +9486,9 @@
       <c r="D140" s="16" t="n"/>
       <c r="E140" s="16" t="n"/>
       <c r="F140" s="16" t="n"/>
+      <c r="G140" s="18" t="n"/>
+      <c r="H140" s="16" t="n"/>
+      <c r="I140" s="16" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="16" t="n"/>
@@ -8768,6 +9497,9 @@
       <c r="D141" s="16" t="n"/>
       <c r="E141" s="16" t="n"/>
       <c r="F141" s="16" t="n"/>
+      <c r="G141" s="18" t="n"/>
+      <c r="H141" s="16" t="n"/>
+      <c r="I141" s="16" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="16" t="n"/>
@@ -8776,6 +9508,9 @@
       <c r="D142" s="16" t="n"/>
       <c r="E142" s="16" t="n"/>
       <c r="F142" s="16" t="n"/>
+      <c r="G142" s="18" t="n"/>
+      <c r="H142" s="16" t="n"/>
+      <c r="I142" s="16" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="16" t="n"/>
@@ -8784,6 +9519,9 @@
       <c r="D143" s="16" t="n"/>
       <c r="E143" s="16" t="n"/>
       <c r="F143" s="16" t="n"/>
+      <c r="G143" s="18" t="n"/>
+      <c r="H143" s="16" t="n"/>
+      <c r="I143" s="16" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="16" t="n"/>
@@ -8792,6 +9530,9 @@
       <c r="D144" s="16" t="n"/>
       <c r="E144" s="16" t="n"/>
       <c r="F144" s="16" t="n"/>
+      <c r="G144" s="18" t="n"/>
+      <c r="H144" s="16" t="n"/>
+      <c r="I144" s="16" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="16" t="n"/>
@@ -8800,6 +9541,9 @@
       <c r="D145" s="16" t="n"/>
       <c r="E145" s="16" t="n"/>
       <c r="F145" s="16" t="n"/>
+      <c r="G145" s="18" t="n"/>
+      <c r="H145" s="16" t="n"/>
+      <c r="I145" s="16" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="16" t="n"/>
@@ -8808,6 +9552,9 @@
       <c r="D146" s="16" t="n"/>
       <c r="E146" s="16" t="n"/>
       <c r="F146" s="16" t="n"/>
+      <c r="G146" s="18" t="n"/>
+      <c r="H146" s="16" t="n"/>
+      <c r="I146" s="16" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="16" t="n"/>
@@ -8816,6 +9563,9 @@
       <c r="D147" s="16" t="n"/>
       <c r="E147" s="16" t="n"/>
       <c r="F147" s="16" t="n"/>
+      <c r="G147" s="18" t="n"/>
+      <c r="H147" s="16" t="n"/>
+      <c r="I147" s="16" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="16" t="n"/>
@@ -8824,6 +9574,9 @@
       <c r="D148" s="16" t="n"/>
       <c r="E148" s="16" t="n"/>
       <c r="F148" s="16" t="n"/>
+      <c r="G148" s="18" t="n"/>
+      <c r="H148" s="16" t="n"/>
+      <c r="I148" s="16" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="16" t="n"/>
@@ -8832,6 +9585,9 @@
       <c r="D149" s="16" t="n"/>
       <c r="E149" s="16" t="n"/>
       <c r="F149" s="16" t="n"/>
+      <c r="G149" s="18" t="n"/>
+      <c r="H149" s="16" t="n"/>
+      <c r="I149" s="16" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="16" t="n"/>
@@ -8840,6 +9596,9 @@
       <c r="D150" s="16" t="n"/>
       <c r="E150" s="16" t="n"/>
       <c r="F150" s="16" t="n"/>
+      <c r="G150" s="18" t="n"/>
+      <c r="H150" s="16" t="n"/>
+      <c r="I150" s="16" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="16" t="n"/>
@@ -8848,6 +9607,9 @@
       <c r="D151" s="16" t="n"/>
       <c r="E151" s="16" t="n"/>
       <c r="F151" s="16" t="n"/>
+      <c r="G151" s="18" t="n"/>
+      <c r="H151" s="16" t="n"/>
+      <c r="I151" s="16" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="16" t="n"/>
@@ -8856,6 +9618,9 @@
       <c r="D152" s="16" t="n"/>
       <c r="E152" s="16" t="n"/>
       <c r="F152" s="16" t="n"/>
+      <c r="G152" s="18" t="n"/>
+      <c r="H152" s="16" t="n"/>
+      <c r="I152" s="16" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="16" t="n"/>
@@ -8864,6 +9629,9 @@
       <c r="D153" s="16" t="n"/>
       <c r="E153" s="16" t="n"/>
       <c r="F153" s="16" t="n"/>
+      <c r="G153" s="18" t="n"/>
+      <c r="H153" s="16" t="n"/>
+      <c r="I153" s="16" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="16" t="n"/>
@@ -8872,6 +9640,9 @@
       <c r="D154" s="16" t="n"/>
       <c r="E154" s="16" t="n"/>
       <c r="F154" s="16" t="n"/>
+      <c r="G154" s="18" t="n"/>
+      <c r="H154" s="16" t="n"/>
+      <c r="I154" s="16" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="16" t="n"/>
@@ -8880,6 +9651,9 @@
       <c r="D155" s="16" t="n"/>
       <c r="E155" s="16" t="n"/>
       <c r="F155" s="16" t="n"/>
+      <c r="G155" s="18" t="n"/>
+      <c r="H155" s="16" t="n"/>
+      <c r="I155" s="16" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="16" t="n"/>
@@ -8888,6 +9662,9 @@
       <c r="D156" s="16" t="n"/>
       <c r="E156" s="16" t="n"/>
       <c r="F156" s="16" t="n"/>
+      <c r="G156" s="18" t="n"/>
+      <c r="H156" s="16" t="n"/>
+      <c r="I156" s="16" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="16" t="n"/>
@@ -8896,6 +9673,9 @@
       <c r="D157" s="16" t="n"/>
       <c r="E157" s="16" t="n"/>
       <c r="F157" s="16" t="n"/>
+      <c r="G157" s="18" t="n"/>
+      <c r="H157" s="16" t="n"/>
+      <c r="I157" s="16" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="16" t="n"/>
@@ -8904,6 +9684,9 @@
       <c r="D158" s="16" t="n"/>
       <c r="E158" s="16" t="n"/>
       <c r="F158" s="16" t="n"/>
+      <c r="G158" s="18" t="n"/>
+      <c r="H158" s="16" t="n"/>
+      <c r="I158" s="16" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="16" t="n"/>
@@ -8912,6 +9695,9 @@
       <c r="D159" s="16" t="n"/>
       <c r="E159" s="16" t="n"/>
       <c r="F159" s="16" t="n"/>
+      <c r="G159" s="18" t="n"/>
+      <c r="H159" s="16" t="n"/>
+      <c r="I159" s="16" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="16" t="n"/>
@@ -8920,6 +9706,9 @@
       <c r="D160" s="16" t="n"/>
       <c r="E160" s="16" t="n"/>
       <c r="F160" s="16" t="n"/>
+      <c r="G160" s="18" t="n"/>
+      <c r="H160" s="16" t="n"/>
+      <c r="I160" s="16" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="16" t="n"/>
@@ -8928,6 +9717,9 @@
       <c r="D161" s="16" t="n"/>
       <c r="E161" s="16" t="n"/>
       <c r="F161" s="16" t="n"/>
+      <c r="G161" s="18" t="n"/>
+      <c r="H161" s="16" t="n"/>
+      <c r="I161" s="16" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="16" t="n"/>
@@ -8936,6 +9728,9 @@
       <c r="D162" s="16" t="n"/>
       <c r="E162" s="16" t="n"/>
       <c r="F162" s="16" t="n"/>
+      <c r="G162" s="18" t="n"/>
+      <c r="H162" s="16" t="n"/>
+      <c r="I162" s="16" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="16" t="n"/>
@@ -8944,6 +9739,9 @@
       <c r="D163" s="16" t="n"/>
       <c r="E163" s="16" t="n"/>
       <c r="F163" s="16" t="n"/>
+      <c r="G163" s="18" t="n"/>
+      <c r="H163" s="16" t="n"/>
+      <c r="I163" s="16" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="16" t="n"/>
@@ -8952,6 +9750,9 @@
       <c r="D164" s="16" t="n"/>
       <c r="E164" s="16" t="n"/>
       <c r="F164" s="16" t="n"/>
+      <c r="G164" s="18" t="n"/>
+      <c r="H164" s="16" t="n"/>
+      <c r="I164" s="16" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="16" t="n"/>
@@ -8960,6 +9761,9 @@
       <c r="D165" s="16" t="n"/>
       <c r="E165" s="16" t="n"/>
       <c r="F165" s="16" t="n"/>
+      <c r="G165" s="18" t="n"/>
+      <c r="H165" s="16" t="n"/>
+      <c r="I165" s="16" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="16" t="n"/>
@@ -8968,6 +9772,9 @@
       <c r="D166" s="16" t="n"/>
       <c r="E166" s="16" t="n"/>
       <c r="F166" s="16" t="n"/>
+      <c r="G166" s="18" t="n"/>
+      <c r="H166" s="16" t="n"/>
+      <c r="I166" s="16" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="16" t="n"/>
@@ -8976,6 +9783,9 @@
       <c r="D167" s="16" t="n"/>
       <c r="E167" s="16" t="n"/>
       <c r="F167" s="16" t="n"/>
+      <c r="G167" s="18" t="n"/>
+      <c r="H167" s="16" t="n"/>
+      <c r="I167" s="16" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="16" t="n"/>
@@ -8984,6 +9794,9 @@
       <c r="D168" s="16" t="n"/>
       <c r="E168" s="16" t="n"/>
       <c r="F168" s="16" t="n"/>
+      <c r="G168" s="18" t="n"/>
+      <c r="H168" s="16" t="n"/>
+      <c r="I168" s="16" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="16" t="n"/>
@@ -8992,6 +9805,9 @@
       <c r="D169" s="16" t="n"/>
       <c r="E169" s="16" t="n"/>
       <c r="F169" s="16" t="n"/>
+      <c r="G169" s="18" t="n"/>
+      <c r="H169" s="16" t="n"/>
+      <c r="I169" s="16" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="16" t="n"/>
@@ -9000,6 +9816,9 @@
       <c r="D170" s="16" t="n"/>
       <c r="E170" s="16" t="n"/>
       <c r="F170" s="16" t="n"/>
+      <c r="G170" s="18" t="n"/>
+      <c r="H170" s="16" t="n"/>
+      <c r="I170" s="16" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="16" t="n"/>
@@ -9008,6 +9827,9 @@
       <c r="D171" s="16" t="n"/>
       <c r="E171" s="16" t="n"/>
       <c r="F171" s="16" t="n"/>
+      <c r="G171" s="18" t="n"/>
+      <c r="H171" s="16" t="n"/>
+      <c r="I171" s="16" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="16" t="n"/>
@@ -9016,6 +9838,9 @@
       <c r="D172" s="16" t="n"/>
       <c r="E172" s="16" t="n"/>
       <c r="F172" s="16" t="n"/>
+      <c r="G172" s="18" t="n"/>
+      <c r="H172" s="16" t="n"/>
+      <c r="I172" s="16" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="16" t="n"/>
@@ -9024,6 +9849,9 @@
       <c r="D173" s="16" t="n"/>
       <c r="E173" s="16" t="n"/>
       <c r="F173" s="16" t="n"/>
+      <c r="G173" s="18" t="n"/>
+      <c r="H173" s="16" t="n"/>
+      <c r="I173" s="16" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="16" t="n"/>
@@ -9032,6 +9860,9 @@
       <c r="D174" s="16" t="n"/>
       <c r="E174" s="16" t="n"/>
       <c r="F174" s="16" t="n"/>
+      <c r="G174" s="18" t="n"/>
+      <c r="H174" s="16" t="n"/>
+      <c r="I174" s="16" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="16" t="n"/>
@@ -9040,6 +9871,9 @@
       <c r="D175" s="16" t="n"/>
       <c r="E175" s="16" t="n"/>
       <c r="F175" s="16" t="n"/>
+      <c r="G175" s="18" t="n"/>
+      <c r="H175" s="16" t="n"/>
+      <c r="I175" s="16" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="16" t="n"/>
@@ -9048,6 +9882,9 @@
       <c r="D176" s="16" t="n"/>
       <c r="E176" s="16" t="n"/>
       <c r="F176" s="16" t="n"/>
+      <c r="G176" s="18" t="n"/>
+      <c r="H176" s="16" t="n"/>
+      <c r="I176" s="16" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="16" t="n"/>
@@ -9056,6 +9893,9 @@
       <c r="D177" s="16" t="n"/>
       <c r="E177" s="16" t="n"/>
       <c r="F177" s="16" t="n"/>
+      <c r="G177" s="18" t="n"/>
+      <c r="H177" s="16" t="n"/>
+      <c r="I177" s="16" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="16" t="n"/>
@@ -9064,6 +9904,9 @@
       <c r="D178" s="16" t="n"/>
       <c r="E178" s="16" t="n"/>
       <c r="F178" s="16" t="n"/>
+      <c r="G178" s="18" t="n"/>
+      <c r="H178" s="16" t="n"/>
+      <c r="I178" s="16" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="16" t="n"/>
@@ -9072,6 +9915,9 @@
       <c r="D179" s="16" t="n"/>
       <c r="E179" s="16" t="n"/>
       <c r="F179" s="16" t="n"/>
+      <c r="G179" s="18" t="n"/>
+      <c r="H179" s="16" t="n"/>
+      <c r="I179" s="16" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="16" t="n"/>
@@ -9080,6 +9926,9 @@
       <c r="D180" s="16" t="n"/>
       <c r="E180" s="16" t="n"/>
       <c r="F180" s="16" t="n"/>
+      <c r="G180" s="18" t="n"/>
+      <c r="H180" s="16" t="n"/>
+      <c r="I180" s="16" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="16" t="n"/>
@@ -9088,6 +9937,9 @@
       <c r="D181" s="16" t="n"/>
       <c r="E181" s="16" t="n"/>
       <c r="F181" s="16" t="n"/>
+      <c r="G181" s="18" t="n"/>
+      <c r="H181" s="16" t="n"/>
+      <c r="I181" s="16" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="16" t="n"/>
@@ -9096,6 +9948,9 @@
       <c r="D182" s="16" t="n"/>
       <c r="E182" s="16" t="n"/>
       <c r="F182" s="16" t="n"/>
+      <c r="G182" s="18" t="n"/>
+      <c r="H182" s="16" t="n"/>
+      <c r="I182" s="16" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="16" t="n"/>
@@ -9104,6 +9959,9 @@
       <c r="D183" s="16" t="n"/>
       <c r="E183" s="16" t="n"/>
       <c r="F183" s="16" t="n"/>
+      <c r="G183" s="18" t="n"/>
+      <c r="H183" s="16" t="n"/>
+      <c r="I183" s="16" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="16" t="n"/>
@@ -9112,6 +9970,9 @@
       <c r="D184" s="16" t="n"/>
       <c r="E184" s="16" t="n"/>
       <c r="F184" s="16" t="n"/>
+      <c r="G184" s="18" t="n"/>
+      <c r="H184" s="16" t="n"/>
+      <c r="I184" s="16" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="16" t="n"/>
@@ -9120,6 +9981,9 @@
       <c r="D185" s="16" t="n"/>
       <c r="E185" s="16" t="n"/>
       <c r="F185" s="16" t="n"/>
+      <c r="G185" s="18" t="n"/>
+      <c r="H185" s="16" t="n"/>
+      <c r="I185" s="16" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="16" t="n"/>
@@ -9128,6 +9992,9 @@
       <c r="D186" s="16" t="n"/>
       <c r="E186" s="16" t="n"/>
       <c r="F186" s="16" t="n"/>
+      <c r="G186" s="18" t="n"/>
+      <c r="H186" s="16" t="n"/>
+      <c r="I186" s="16" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="16" t="n"/>
@@ -9136,6 +10003,9 @@
       <c r="D187" s="16" t="n"/>
       <c r="E187" s="16" t="n"/>
       <c r="F187" s="16" t="n"/>
+      <c r="G187" s="18" t="n"/>
+      <c r="H187" s="16" t="n"/>
+      <c r="I187" s="16" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="16" t="n"/>
@@ -9144,6 +10014,9 @@
       <c r="D188" s="16" t="n"/>
       <c r="E188" s="16" t="n"/>
       <c r="F188" s="16" t="n"/>
+      <c r="G188" s="18" t="n"/>
+      <c r="H188" s="16" t="n"/>
+      <c r="I188" s="16" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="16" t="n"/>
@@ -9152,6 +10025,9 @@
       <c r="D189" s="16" t="n"/>
       <c r="E189" s="16" t="n"/>
       <c r="F189" s="16" t="n"/>
+      <c r="G189" s="18" t="n"/>
+      <c r="H189" s="16" t="n"/>
+      <c r="I189" s="16" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="16" t="n"/>
@@ -9160,6 +10036,9 @@
       <c r="D190" s="16" t="n"/>
       <c r="E190" s="16" t="n"/>
       <c r="F190" s="16" t="n"/>
+      <c r="G190" s="18" t="n"/>
+      <c r="H190" s="16" t="n"/>
+      <c r="I190" s="16" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="16" t="n"/>
@@ -9168,6 +10047,9 @@
       <c r="D191" s="16" t="n"/>
       <c r="E191" s="16" t="n"/>
       <c r="F191" s="16" t="n"/>
+      <c r="G191" s="18" t="n"/>
+      <c r="H191" s="16" t="n"/>
+      <c r="I191" s="16" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="16" t="n"/>
@@ -9176,6 +10058,9 @@
       <c r="D192" s="16" t="n"/>
       <c r="E192" s="16" t="n"/>
       <c r="F192" s="16" t="n"/>
+      <c r="G192" s="18" t="n"/>
+      <c r="H192" s="16" t="n"/>
+      <c r="I192" s="16" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="16" t="n"/>
@@ -9184,6 +10069,9 @@
       <c r="D193" s="16" t="n"/>
       <c r="E193" s="16" t="n"/>
       <c r="F193" s="16" t="n"/>
+      <c r="G193" s="18" t="n"/>
+      <c r="H193" s="16" t="n"/>
+      <c r="I193" s="16" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="16" t="n"/>
@@ -9192,6 +10080,9 @@
       <c r="D194" s="16" t="n"/>
       <c r="E194" s="16" t="n"/>
       <c r="F194" s="16" t="n"/>
+      <c r="G194" s="18" t="n"/>
+      <c r="H194" s="16" t="n"/>
+      <c r="I194" s="16" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="16" t="n"/>
@@ -9200,6 +10091,9 @@
       <c r="D195" s="16" t="n"/>
       <c r="E195" s="16" t="n"/>
       <c r="F195" s="16" t="n"/>
+      <c r="G195" s="18" t="n"/>
+      <c r="H195" s="16" t="n"/>
+      <c r="I195" s="16" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="16" t="n"/>
@@ -9208,6 +10102,9 @@
       <c r="D196" s="16" t="n"/>
       <c r="E196" s="16" t="n"/>
       <c r="F196" s="16" t="n"/>
+      <c r="G196" s="18" t="n"/>
+      <c r="H196" s="16" t="n"/>
+      <c r="I196" s="16" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="16" t="n"/>
@@ -9216,6 +10113,9 @@
       <c r="D197" s="16" t="n"/>
       <c r="E197" s="16" t="n"/>
       <c r="F197" s="16" t="n"/>
+      <c r="G197" s="18" t="n"/>
+      <c r="H197" s="16" t="n"/>
+      <c r="I197" s="16" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="16" t="n"/>
@@ -9224,6 +10124,9 @@
       <c r="D198" s="16" t="n"/>
       <c r="E198" s="16" t="n"/>
       <c r="F198" s="16" t="n"/>
+      <c r="G198" s="18" t="n"/>
+      <c r="H198" s="16" t="n"/>
+      <c r="I198" s="16" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="16" t="n"/>
@@ -9232,6 +10135,9 @@
       <c r="D199" s="16" t="n"/>
       <c r="E199" s="16" t="n"/>
       <c r="F199" s="16" t="n"/>
+      <c r="G199" s="18" t="n"/>
+      <c r="H199" s="16" t="n"/>
+      <c r="I199" s="16" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="16" t="n"/>
@@ -9240,6 +10146,9 @@
       <c r="D200" s="16" t="n"/>
       <c r="E200" s="16" t="n"/>
       <c r="F200" s="16" t="n"/>
+      <c r="G200" s="18" t="n"/>
+      <c r="H200" s="16" t="n"/>
+      <c r="I200" s="16" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="16" t="n"/>
@@ -9248,6 +10157,9 @@
       <c r="D201" s="16" t="n"/>
       <c r="E201" s="16" t="n"/>
       <c r="F201" s="16" t="n"/>
+      <c r="G201" s="18" t="n"/>
+      <c r="H201" s="16" t="n"/>
+      <c r="I201" s="16" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Order column for milestones; AVD milestone order
</commit_message>
<xml_diff>
--- a/data/roadmaps/Roadmap - Combined.xlsx
+++ b/data/roadmaps/Roadmap - Combined.xlsx
@@ -1015,7 +1015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O201"/>
+  <dimension ref="A1:P201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1033,6 +1033,7 @@
     <col width="40" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="48" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1111,6 +1112,11 @@
           <t>Notes (not shown on dashboard)</t>
         </is>
       </c>
+      <c r="P1" s="12" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -1174,6 +1180,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Tracking SPA-2583 (AI Search, SM approved) and SPA-2589 (Doc Intelligence, SSO review). Source: COMET&lt;&gt;CMS PO updates 9/16, 9/23, 10/7.</t>
         </is>
       </c>
+      <c r="P2" s="13" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -1229,6 +1236,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Initial planning/discovery noted 9/16; MSFT demo held 9/24; follow-up meeting pending (10/7). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P3" s="13" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -1292,6 +1300,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. SIA raised by 9/23. Source: COMET&lt;&gt;CMS PO updates 9/23, 10/7.</t>
         </is>
       </c>
+      <c r="P4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -1347,6 +1356,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Zscaler and Centralized Firewall EOC integration completed (reported 9/09). Remaining services not listed in the updates. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P5" s="13" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -1402,6 +1412,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Being tracked in the IUSG weekly call; no committed timeline yet. Source: COMET&lt;&gt;CMS PO updates 9/16, 9/23, 10/7.</t>
         </is>
       </c>
+      <c r="P6" s="13" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -1457,6 +1468,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. New provisioning workflow verified (reported 9/16). Next step after verification not stated. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -1512,6 +1524,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Ongoing handoff. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P8" s="13" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -1567,6 +1580,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Reported PROD Ready by 9/16. EQRS will need to move to the revised access management approach later (see GCP-08). Source: COMET&lt;&gt;CMS PO updates 9/16-10/7.</t>
         </is>
       </c>
+      <c r="P9" s="13" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -1630,6 +1644,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Open SIAs on 10/7: Service Directory CLDSPT-114389 (ON HOLD), Cloud Build CLDSPT-112641 (ON HOLD), Workflows API CLDSPT-115742 (ON HOLD), Knowledge Catalog CLDSPT-115656 (backlog), VM Migration CLDSPT-116513 (backlog). All but VM Migration are enabled in ADO non-prod with ADO ISSO/BO approval. 9/16: Parameter Manager, Database Migration Service and Storage Transfer not approved at GSS level; ADOs may enable in their own boundary with ISSO/BO risk acceptance. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P10" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -1693,6 +1708,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. ONBI-14306 tenant provisioning DONE; CPT-6984 funding APPROVED; project created (FY26INIT-1176 IN PROGRESS); CLDSPT-116097 Snowflake connectivity RESOLVED; Knowledge Catalog SIA CLDSPT-115656 in backlog. Source: COMET&lt;&gt;CMS PO updates 9/23, 10/7.</t>
         </is>
       </c>
+      <c r="P11" s="13" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -1752,6 +1768,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. ONBI-14712 tenant provisioning DONE; CLDSPT-116263 project created, testing network before handover. Source: COMET&lt;&gt;CMS PO updates 10/7.</t>
         </is>
       </c>
+      <c r="P12" s="13" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -1811,6 +1828,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Scripts integrated with the SPA workflow and being tested (9/23, 10/7). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P13" s="13" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -1870,6 +1888,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. FY26INIT-1084 still TO DO on 10/7. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P14" s="13" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -1925,6 +1944,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Zscaler and Centralized Firewall done; remaining services not listed. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -1980,6 +2000,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Workflow validated; EQRS migration still to come. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -2035,6 +2056,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Hot item 10/7: finalizing region; stakeholder meeting with Chris Vee on 10/13. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P17" s="13" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -2090,6 +2112,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. FY26INIT-1097 unified docs DONE (9/23); CCG updates with COMMS ongoing. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P18" s="13" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -2149,6 +2172,7 @@
           <t>Start date placeholder. Target moved 8/31 (9/16 update) -&gt; 9/30 (9/23) -&gt; 10/15 (10/7). SMTP production ready 10/7; backup functions completed 10/7 (prod function pending). Custom Software Source fix in OS Management Hub 3.8 (Oracle support case). Internal DNS testing was blocked on a security change request (9/16). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
@@ -2208,6 +2232,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Oracle to give updated ETA (logging), confirm roadmap (reboot), explore earlier release (patching). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P20" s="13" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
@@ -2263,6 +2288,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. SecOps confirmed functioning (9/23, 10/7); minor field sorting tweaks need SOC input. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P21" s="13" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -2318,6 +2344,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Being evaluated in the non-prod connectivity compartment (10/7). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P22" s="13" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
@@ -2377,6 +2404,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Security review defined compliance boundary; shared GSS compartment approved (CLDSPT-115520); logging VCN and Cloudflare VPN created, testing pending; DOOM access granted (CLDSPT-115181). Open question: does the tenancy support all logging services, or is a new subscription (CPT approval) needed? Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P23" s="13" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
@@ -2436,6 +2464,7 @@
           <t>Start date placeholder. Dates moved: EUA/EFT migrations 9/18 -&gt; TBD; process doc 9/21 -&gt; 9/30 -&gt; 10/26; shared services 9/30 -&gt; 10/30; MiSP non-prod onboarding 9/25 -&gt; TBD. Oracle SRs 4-0003803176 (resolved) and 4-0003830164 (under review). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
@@ -2491,6 +2520,7 @@
           <t>Start date placeholder. Network installation and onsite validation started (9/23). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
@@ -2550,6 +2580,9 @@
           <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
       </c>
+      <c r="P26" s="13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
@@ -2608,6 +2641,9 @@
         <is>
           <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
+      </c>
+      <c r="P27" s="13" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -2664,6 +2700,9 @@
           <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
       </c>
+      <c r="P28" s="13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
@@ -2719,6 +2758,9 @@
           <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
       </c>
+      <c r="P29" s="13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
@@ -2777,6 +2819,9 @@
         <is>
           <t>Source: AVD FY27 Milestones page (19 Oct 2026) via AVD FY27 Roadmap DRAFT 2. Status and theme are not in the source; carried over from the 10/7 PO update - confirm with the DM.</t>
         </is>
+      </c>
+      <c r="P30" s="13" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -2833,6 +2878,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. First iteration (ELB) 9/23; consolidated AWS CloudFront + ELB dashboard with listener and cipher columns 10/7. Next: TLS version and cipher filters; Azure and GCP dashboards; on-prem needs Splunk DC access and federated search. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P31" s="13" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
@@ -2888,6 +2934,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Kickoff 9/16; S3 bucket and IAM role delivered 9/23; export landing in Observability Hub account 10/7. Next: ingest and build lookup table, then a simple IP lookup app. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P32" s="13" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
@@ -2943,6 +2990,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Non-descriptive fields traced to Cribl Search normalizing only for Splunk Cloud, not ITOPS; MiSP normalized both. CCG for Azure/GCP custom log collection pending COMMS review and CMS approval. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P33" s="13" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
@@ -2998,6 +3046,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. SplunkPS delivered its estimate to Chris V. (by 10/7). Waiting on MiSP for ITOPS and DC costs. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P34" s="13" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
@@ -3053,6 +3102,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. SDL started GCP flow log ingestion (10/7); SDL plans an instance in GCP (funding to check). Also: route VPC flow logs to Cribl with MiSP; centralized OCI Object Storage with the OCI team. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P35" s="13" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
@@ -3108,6 +3158,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Service account received; CCIC/SOC installing JRE prerequisites (10/7). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P36" s="13" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
@@ -3167,6 +3218,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Draft roadmap done (9/09); depends on the Cribl task for routing AWS logs. Open question: who owns ES and Core (POC/responsibility). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P37" s="13" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
@@ -3222,6 +3274,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. AD (Outpost) onboarded (9/16); SMTP (Outpost) onboarded (by 9/23); SRE onboarding 6 MEF apps (APS, eCHIMP, MARx, MEPBS, NGD, NPPES); teams asked to update Datadog tags. Source: COMET&lt;&gt;CMS PO updates (PI-2 plan).</t>
         </is>
       </c>
+      <c r="P38" s="13" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
@@ -3277,6 +3330,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Drafts with COMMS; publishing in progress (9/23, 10/7). Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P39" s="13" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
@@ -3340,6 +3394,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. Azure solution developed, validation pending. GCP solution deployment by MiSP (DOOMS) to one account waiting on the Cloud Build SIA. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P40" s="13" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
@@ -3395,6 +3450,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. BaseCAMP data in ObsHub and first lookup table (9/16); two tables created (by 9/23); next: apply to EOC dashboard. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P41" s="13" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
@@ -3450,6 +3506,7 @@
           <t>Start/end dates are placeholders (not in the updates); confirm with the PO. MiSP finished evaluating Cribl Replay; demo session pending. Source: COMET&lt;&gt;CMS PO updates.</t>
         </is>
       </c>
+      <c r="P42" s="13" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="n"/>
@@ -3467,6 +3524,7 @@
       <c r="M43" s="17" t="n"/>
       <c r="N43" s="18" t="n"/>
       <c r="O43" s="17" t="n"/>
+      <c r="P43" s="16" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="16" t="n"/>
@@ -3484,6 +3542,7 @@
       <c r="M44" s="17" t="n"/>
       <c r="N44" s="18" t="n"/>
       <c r="O44" s="17" t="n"/>
+      <c r="P44" s="16" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="16" t="n"/>
@@ -3501,6 +3560,7 @@
       <c r="M45" s="17" t="n"/>
       <c r="N45" s="18" t="n"/>
       <c r="O45" s="17" t="n"/>
+      <c r="P45" s="16" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="16" t="n"/>
@@ -3518,6 +3578,7 @@
       <c r="M46" s="17" t="n"/>
       <c r="N46" s="18" t="n"/>
       <c r="O46" s="17" t="n"/>
+      <c r="P46" s="16" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="n"/>
@@ -3535,6 +3596,7 @@
       <c r="M47" s="17" t="n"/>
       <c r="N47" s="18" t="n"/>
       <c r="O47" s="17" t="n"/>
+      <c r="P47" s="16" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="16" t="n"/>
@@ -3552,6 +3614,7 @@
       <c r="M48" s="17" t="n"/>
       <c r="N48" s="18" t="n"/>
       <c r="O48" s="17" t="n"/>
+      <c r="P48" s="16" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="n"/>
@@ -3569,6 +3632,7 @@
       <c r="M49" s="17" t="n"/>
       <c r="N49" s="18" t="n"/>
       <c r="O49" s="17" t="n"/>
+      <c r="P49" s="16" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="n"/>
@@ -3586,6 +3650,7 @@
       <c r="M50" s="17" t="n"/>
       <c r="N50" s="18" t="n"/>
       <c r="O50" s="17" t="n"/>
+      <c r="P50" s="16" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="n"/>
@@ -3603,6 +3668,7 @@
       <c r="M51" s="17" t="n"/>
       <c r="N51" s="18" t="n"/>
       <c r="O51" s="17" t="n"/>
+      <c r="P51" s="16" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="16" t="n"/>
@@ -3620,6 +3686,7 @@
       <c r="M52" s="17" t="n"/>
       <c r="N52" s="18" t="n"/>
       <c r="O52" s="17" t="n"/>
+      <c r="P52" s="16" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="16" t="n"/>
@@ -3637,6 +3704,7 @@
       <c r="M53" s="17" t="n"/>
       <c r="N53" s="18" t="n"/>
       <c r="O53" s="17" t="n"/>
+      <c r="P53" s="16" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="16" t="n"/>
@@ -3654,6 +3722,7 @@
       <c r="M54" s="17" t="n"/>
       <c r="N54" s="18" t="n"/>
       <c r="O54" s="17" t="n"/>
+      <c r="P54" s="16" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="16" t="n"/>
@@ -3671,6 +3740,7 @@
       <c r="M55" s="17" t="n"/>
       <c r="N55" s="18" t="n"/>
       <c r="O55" s="17" t="n"/>
+      <c r="P55" s="16" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="n"/>
@@ -3688,6 +3758,7 @@
       <c r="M56" s="17" t="n"/>
       <c r="N56" s="18" t="n"/>
       <c r="O56" s="17" t="n"/>
+      <c r="P56" s="16" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="16" t="n"/>
@@ -3705,6 +3776,7 @@
       <c r="M57" s="17" t="n"/>
       <c r="N57" s="18" t="n"/>
       <c r="O57" s="17" t="n"/>
+      <c r="P57" s="16" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="16" t="n"/>
@@ -3722,6 +3794,7 @@
       <c r="M58" s="17" t="n"/>
       <c r="N58" s="18" t="n"/>
       <c r="O58" s="17" t="n"/>
+      <c r="P58" s="16" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="16" t="n"/>
@@ -3739,6 +3812,7 @@
       <c r="M59" s="17" t="n"/>
       <c r="N59" s="18" t="n"/>
       <c r="O59" s="17" t="n"/>
+      <c r="P59" s="16" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="n"/>
@@ -3756,6 +3830,7 @@
       <c r="M60" s="17" t="n"/>
       <c r="N60" s="18" t="n"/>
       <c r="O60" s="17" t="n"/>
+      <c r="P60" s="16" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="n"/>
@@ -3773,6 +3848,7 @@
       <c r="M61" s="17" t="n"/>
       <c r="N61" s="18" t="n"/>
       <c r="O61" s="17" t="n"/>
+      <c r="P61" s="16" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="16" t="n"/>
@@ -3790,6 +3866,7 @@
       <c r="M62" s="17" t="n"/>
       <c r="N62" s="18" t="n"/>
       <c r="O62" s="17" t="n"/>
+      <c r="P62" s="16" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="16" t="n"/>
@@ -3807,6 +3884,7 @@
       <c r="M63" s="17" t="n"/>
       <c r="N63" s="18" t="n"/>
       <c r="O63" s="17" t="n"/>
+      <c r="P63" s="16" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="16" t="n"/>
@@ -3824,6 +3902,7 @@
       <c r="M64" s="17" t="n"/>
       <c r="N64" s="18" t="n"/>
       <c r="O64" s="17" t="n"/>
+      <c r="P64" s="16" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="16" t="n"/>
@@ -3841,6 +3920,7 @@
       <c r="M65" s="17" t="n"/>
       <c r="N65" s="18" t="n"/>
       <c r="O65" s="17" t="n"/>
+      <c r="P65" s="16" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="16" t="n"/>
@@ -3858,6 +3938,7 @@
       <c r="M66" s="17" t="n"/>
       <c r="N66" s="18" t="n"/>
       <c r="O66" s="17" t="n"/>
+      <c r="P66" s="16" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="16" t="n"/>
@@ -3875,6 +3956,7 @@
       <c r="M67" s="17" t="n"/>
       <c r="N67" s="18" t="n"/>
       <c r="O67" s="17" t="n"/>
+      <c r="P67" s="16" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="n"/>
@@ -3892,6 +3974,7 @@
       <c r="M68" s="17" t="n"/>
       <c r="N68" s="18" t="n"/>
       <c r="O68" s="17" t="n"/>
+      <c r="P68" s="16" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="n"/>
@@ -3909,6 +3992,7 @@
       <c r="M69" s="17" t="n"/>
       <c r="N69" s="18" t="n"/>
       <c r="O69" s="17" t="n"/>
+      <c r="P69" s="16" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="16" t="n"/>
@@ -3926,6 +4010,7 @@
       <c r="M70" s="17" t="n"/>
       <c r="N70" s="18" t="n"/>
       <c r="O70" s="17" t="n"/>
+      <c r="P70" s="16" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="16" t="n"/>
@@ -3943,6 +4028,7 @@
       <c r="M71" s="17" t="n"/>
       <c r="N71" s="18" t="n"/>
       <c r="O71" s="17" t="n"/>
+      <c r="P71" s="16" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="16" t="n"/>
@@ -3960,6 +4046,7 @@
       <c r="M72" s="17" t="n"/>
       <c r="N72" s="18" t="n"/>
       <c r="O72" s="17" t="n"/>
+      <c r="P72" s="16" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="16" t="n"/>
@@ -3977,6 +4064,7 @@
       <c r="M73" s="17" t="n"/>
       <c r="N73" s="18" t="n"/>
       <c r="O73" s="17" t="n"/>
+      <c r="P73" s="16" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="16" t="n"/>
@@ -3994,6 +4082,7 @@
       <c r="M74" s="17" t="n"/>
       <c r="N74" s="18" t="n"/>
       <c r="O74" s="17" t="n"/>
+      <c r="P74" s="16" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="16" t="n"/>
@@ -4011,6 +4100,7 @@
       <c r="M75" s="17" t="n"/>
       <c r="N75" s="18" t="n"/>
       <c r="O75" s="17" t="n"/>
+      <c r="P75" s="16" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="16" t="n"/>
@@ -4028,6 +4118,7 @@
       <c r="M76" s="17" t="n"/>
       <c r="N76" s="18" t="n"/>
       <c r="O76" s="17" t="n"/>
+      <c r="P76" s="16" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="16" t="n"/>
@@ -4045,6 +4136,7 @@
       <c r="M77" s="17" t="n"/>
       <c r="N77" s="18" t="n"/>
       <c r="O77" s="17" t="n"/>
+      <c r="P77" s="16" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="16" t="n"/>
@@ -4062,6 +4154,7 @@
       <c r="M78" s="17" t="n"/>
       <c r="N78" s="18" t="n"/>
       <c r="O78" s="17" t="n"/>
+      <c r="P78" s="16" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="16" t="n"/>
@@ -4079,6 +4172,7 @@
       <c r="M79" s="17" t="n"/>
       <c r="N79" s="18" t="n"/>
       <c r="O79" s="17" t="n"/>
+      <c r="P79" s="16" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="16" t="n"/>
@@ -4096,6 +4190,7 @@
       <c r="M80" s="17" t="n"/>
       <c r="N80" s="18" t="n"/>
       <c r="O80" s="17" t="n"/>
+      <c r="P80" s="16" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="16" t="n"/>
@@ -4113,6 +4208,7 @@
       <c r="M81" s="17" t="n"/>
       <c r="N81" s="18" t="n"/>
       <c r="O81" s="17" t="n"/>
+      <c r="P81" s="16" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="16" t="n"/>
@@ -4130,6 +4226,7 @@
       <c r="M82" s="17" t="n"/>
       <c r="N82" s="18" t="n"/>
       <c r="O82" s="17" t="n"/>
+      <c r="P82" s="16" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="16" t="n"/>
@@ -4147,6 +4244,7 @@
       <c r="M83" s="17" t="n"/>
       <c r="N83" s="18" t="n"/>
       <c r="O83" s="17" t="n"/>
+      <c r="P83" s="16" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="16" t="n"/>
@@ -4164,6 +4262,7 @@
       <c r="M84" s="17" t="n"/>
       <c r="N84" s="18" t="n"/>
       <c r="O84" s="17" t="n"/>
+      <c r="P84" s="16" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="16" t="n"/>
@@ -4181,6 +4280,7 @@
       <c r="M85" s="17" t="n"/>
       <c r="N85" s="18" t="n"/>
       <c r="O85" s="17" t="n"/>
+      <c r="P85" s="16" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="16" t="n"/>
@@ -4198,6 +4298,7 @@
       <c r="M86" s="17" t="n"/>
       <c r="N86" s="18" t="n"/>
       <c r="O86" s="17" t="n"/>
+      <c r="P86" s="16" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="16" t="n"/>
@@ -4215,6 +4316,7 @@
       <c r="M87" s="17" t="n"/>
       <c r="N87" s="18" t="n"/>
       <c r="O87" s="17" t="n"/>
+      <c r="P87" s="16" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="16" t="n"/>
@@ -4232,6 +4334,7 @@
       <c r="M88" s="17" t="n"/>
       <c r="N88" s="18" t="n"/>
       <c r="O88" s="17" t="n"/>
+      <c r="P88" s="16" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="16" t="n"/>
@@ -4249,6 +4352,7 @@
       <c r="M89" s="17" t="n"/>
       <c r="N89" s="18" t="n"/>
       <c r="O89" s="17" t="n"/>
+      <c r="P89" s="16" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="16" t="n"/>
@@ -4266,6 +4370,7 @@
       <c r="M90" s="17" t="n"/>
       <c r="N90" s="18" t="n"/>
       <c r="O90" s="17" t="n"/>
+      <c r="P90" s="16" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="16" t="n"/>
@@ -4283,6 +4388,7 @@
       <c r="M91" s="17" t="n"/>
       <c r="N91" s="18" t="n"/>
       <c r="O91" s="17" t="n"/>
+      <c r="P91" s="16" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="16" t="n"/>
@@ -4300,6 +4406,7 @@
       <c r="M92" s="17" t="n"/>
       <c r="N92" s="18" t="n"/>
       <c r="O92" s="17" t="n"/>
+      <c r="P92" s="16" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="16" t="n"/>
@@ -4317,6 +4424,7 @@
       <c r="M93" s="17" t="n"/>
       <c r="N93" s="18" t="n"/>
       <c r="O93" s="17" t="n"/>
+      <c r="P93" s="16" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="16" t="n"/>
@@ -4334,6 +4442,7 @@
       <c r="M94" s="17" t="n"/>
       <c r="N94" s="18" t="n"/>
       <c r="O94" s="17" t="n"/>
+      <c r="P94" s="16" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="16" t="n"/>
@@ -4351,6 +4460,7 @@
       <c r="M95" s="17" t="n"/>
       <c r="N95" s="18" t="n"/>
       <c r="O95" s="17" t="n"/>
+      <c r="P95" s="16" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="16" t="n"/>
@@ -4368,6 +4478,7 @@
       <c r="M96" s="17" t="n"/>
       <c r="N96" s="18" t="n"/>
       <c r="O96" s="17" t="n"/>
+      <c r="P96" s="16" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="16" t="n"/>
@@ -4385,6 +4496,7 @@
       <c r="M97" s="17" t="n"/>
       <c r="N97" s="18" t="n"/>
       <c r="O97" s="17" t="n"/>
+      <c r="P97" s="16" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="16" t="n"/>
@@ -4402,6 +4514,7 @@
       <c r="M98" s="17" t="n"/>
       <c r="N98" s="18" t="n"/>
       <c r="O98" s="17" t="n"/>
+      <c r="P98" s="16" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="16" t="n"/>
@@ -4419,6 +4532,7 @@
       <c r="M99" s="17" t="n"/>
       <c r="N99" s="18" t="n"/>
       <c r="O99" s="17" t="n"/>
+      <c r="P99" s="16" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="16" t="n"/>
@@ -4436,6 +4550,7 @@
       <c r="M100" s="17" t="n"/>
       <c r="N100" s="18" t="n"/>
       <c r="O100" s="17" t="n"/>
+      <c r="P100" s="16" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="16" t="n"/>
@@ -4453,6 +4568,7 @@
       <c r="M101" s="17" t="n"/>
       <c r="N101" s="18" t="n"/>
       <c r="O101" s="17" t="n"/>
+      <c r="P101" s="16" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="16" t="n"/>
@@ -4470,6 +4586,7 @@
       <c r="M102" s="17" t="n"/>
       <c r="N102" s="18" t="n"/>
       <c r="O102" s="17" t="n"/>
+      <c r="P102" s="16" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="16" t="n"/>
@@ -4487,6 +4604,7 @@
       <c r="M103" s="17" t="n"/>
       <c r="N103" s="18" t="n"/>
       <c r="O103" s="17" t="n"/>
+      <c r="P103" s="16" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="16" t="n"/>
@@ -4504,6 +4622,7 @@
       <c r="M104" s="17" t="n"/>
       <c r="N104" s="18" t="n"/>
       <c r="O104" s="17" t="n"/>
+      <c r="P104" s="16" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="16" t="n"/>
@@ -4521,6 +4640,7 @@
       <c r="M105" s="17" t="n"/>
       <c r="N105" s="18" t="n"/>
       <c r="O105" s="17" t="n"/>
+      <c r="P105" s="16" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="16" t="n"/>
@@ -4538,6 +4658,7 @@
       <c r="M106" s="17" t="n"/>
       <c r="N106" s="18" t="n"/>
       <c r="O106" s="17" t="n"/>
+      <c r="P106" s="16" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="16" t="n"/>
@@ -4555,6 +4676,7 @@
       <c r="M107" s="17" t="n"/>
       <c r="N107" s="18" t="n"/>
       <c r="O107" s="17" t="n"/>
+      <c r="P107" s="16" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="16" t="n"/>
@@ -4572,6 +4694,7 @@
       <c r="M108" s="17" t="n"/>
       <c r="N108" s="18" t="n"/>
       <c r="O108" s="17" t="n"/>
+      <c r="P108" s="16" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="16" t="n"/>
@@ -4589,6 +4712,7 @@
       <c r="M109" s="17" t="n"/>
       <c r="N109" s="18" t="n"/>
       <c r="O109" s="17" t="n"/>
+      <c r="P109" s="16" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="16" t="n"/>
@@ -4606,6 +4730,7 @@
       <c r="M110" s="17" t="n"/>
       <c r="N110" s="18" t="n"/>
       <c r="O110" s="17" t="n"/>
+      <c r="P110" s="16" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="16" t="n"/>
@@ -4623,6 +4748,7 @@
       <c r="M111" s="17" t="n"/>
       <c r="N111" s="18" t="n"/>
       <c r="O111" s="17" t="n"/>
+      <c r="P111" s="16" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="16" t="n"/>
@@ -4640,6 +4766,7 @@
       <c r="M112" s="17" t="n"/>
       <c r="N112" s="18" t="n"/>
       <c r="O112" s="17" t="n"/>
+      <c r="P112" s="16" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="16" t="n"/>
@@ -4657,6 +4784,7 @@
       <c r="M113" s="17" t="n"/>
       <c r="N113" s="18" t="n"/>
       <c r="O113" s="17" t="n"/>
+      <c r="P113" s="16" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="16" t="n"/>
@@ -4674,6 +4802,7 @@
       <c r="M114" s="17" t="n"/>
       <c r="N114" s="18" t="n"/>
       <c r="O114" s="17" t="n"/>
+      <c r="P114" s="16" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="16" t="n"/>
@@ -4691,6 +4820,7 @@
       <c r="M115" s="17" t="n"/>
       <c r="N115" s="18" t="n"/>
       <c r="O115" s="17" t="n"/>
+      <c r="P115" s="16" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="16" t="n"/>
@@ -4708,6 +4838,7 @@
       <c r="M116" s="17" t="n"/>
       <c r="N116" s="18" t="n"/>
       <c r="O116" s="17" t="n"/>
+      <c r="P116" s="16" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="16" t="n"/>
@@ -4725,6 +4856,7 @@
       <c r="M117" s="17" t="n"/>
       <c r="N117" s="18" t="n"/>
       <c r="O117" s="17" t="n"/>
+      <c r="P117" s="16" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="16" t="n"/>
@@ -4742,6 +4874,7 @@
       <c r="M118" s="17" t="n"/>
       <c r="N118" s="18" t="n"/>
       <c r="O118" s="17" t="n"/>
+      <c r="P118" s="16" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="16" t="n"/>
@@ -4759,6 +4892,7 @@
       <c r="M119" s="17" t="n"/>
       <c r="N119" s="18" t="n"/>
       <c r="O119" s="17" t="n"/>
+      <c r="P119" s="16" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="16" t="n"/>
@@ -4776,6 +4910,7 @@
       <c r="M120" s="17" t="n"/>
       <c r="N120" s="18" t="n"/>
       <c r="O120" s="17" t="n"/>
+      <c r="P120" s="16" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="16" t="n"/>
@@ -4793,6 +4928,7 @@
       <c r="M121" s="17" t="n"/>
       <c r="N121" s="18" t="n"/>
       <c r="O121" s="17" t="n"/>
+      <c r="P121" s="16" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="16" t="n"/>
@@ -4810,6 +4946,7 @@
       <c r="M122" s="17" t="n"/>
       <c r="N122" s="18" t="n"/>
       <c r="O122" s="17" t="n"/>
+      <c r="P122" s="16" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="16" t="n"/>
@@ -4827,6 +4964,7 @@
       <c r="M123" s="17" t="n"/>
       <c r="N123" s="18" t="n"/>
       <c r="O123" s="17" t="n"/>
+      <c r="P123" s="16" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="16" t="n"/>
@@ -4844,6 +4982,7 @@
       <c r="M124" s="17" t="n"/>
       <c r="N124" s="18" t="n"/>
       <c r="O124" s="17" t="n"/>
+      <c r="P124" s="16" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="16" t="n"/>
@@ -4861,6 +5000,7 @@
       <c r="M125" s="17" t="n"/>
       <c r="N125" s="18" t="n"/>
       <c r="O125" s="17" t="n"/>
+      <c r="P125" s="16" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="16" t="n"/>
@@ -4878,6 +5018,7 @@
       <c r="M126" s="17" t="n"/>
       <c r="N126" s="18" t="n"/>
       <c r="O126" s="17" t="n"/>
+      <c r="P126" s="16" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="16" t="n"/>
@@ -4895,6 +5036,7 @@
       <c r="M127" s="17" t="n"/>
       <c r="N127" s="18" t="n"/>
       <c r="O127" s="17" t="n"/>
+      <c r="P127" s="16" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="16" t="n"/>
@@ -4912,6 +5054,7 @@
       <c r="M128" s="17" t="n"/>
       <c r="N128" s="18" t="n"/>
       <c r="O128" s="17" t="n"/>
+      <c r="P128" s="16" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="16" t="n"/>
@@ -4929,6 +5072,7 @@
       <c r="M129" s="17" t="n"/>
       <c r="N129" s="18" t="n"/>
       <c r="O129" s="17" t="n"/>
+      <c r="P129" s="16" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="16" t="n"/>
@@ -4946,6 +5090,7 @@
       <c r="M130" s="17" t="n"/>
       <c r="N130" s="18" t="n"/>
       <c r="O130" s="17" t="n"/>
+      <c r="P130" s="16" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="16" t="n"/>
@@ -4963,6 +5108,7 @@
       <c r="M131" s="17" t="n"/>
       <c r="N131" s="18" t="n"/>
       <c r="O131" s="17" t="n"/>
+      <c r="P131" s="16" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="16" t="n"/>
@@ -4980,6 +5126,7 @@
       <c r="M132" s="17" t="n"/>
       <c r="N132" s="18" t="n"/>
       <c r="O132" s="17" t="n"/>
+      <c r="P132" s="16" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="16" t="n"/>
@@ -4997,6 +5144,7 @@
       <c r="M133" s="17" t="n"/>
       <c r="N133" s="18" t="n"/>
       <c r="O133" s="17" t="n"/>
+      <c r="P133" s="16" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="16" t="n"/>
@@ -5014,6 +5162,7 @@
       <c r="M134" s="17" t="n"/>
       <c r="N134" s="18" t="n"/>
       <c r="O134" s="17" t="n"/>
+      <c r="P134" s="16" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="16" t="n"/>
@@ -5031,6 +5180,7 @@
       <c r="M135" s="17" t="n"/>
       <c r="N135" s="18" t="n"/>
       <c r="O135" s="17" t="n"/>
+      <c r="P135" s="16" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="16" t="n"/>
@@ -5048,6 +5198,7 @@
       <c r="M136" s="17" t="n"/>
       <c r="N136" s="18" t="n"/>
       <c r="O136" s="17" t="n"/>
+      <c r="P136" s="16" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="16" t="n"/>
@@ -5065,6 +5216,7 @@
       <c r="M137" s="17" t="n"/>
       <c r="N137" s="18" t="n"/>
       <c r="O137" s="17" t="n"/>
+      <c r="P137" s="16" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="16" t="n"/>
@@ -5082,6 +5234,7 @@
       <c r="M138" s="17" t="n"/>
       <c r="N138" s="18" t="n"/>
       <c r="O138" s="17" t="n"/>
+      <c r="P138" s="16" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="16" t="n"/>
@@ -5099,6 +5252,7 @@
       <c r="M139" s="17" t="n"/>
       <c r="N139" s="18" t="n"/>
       <c r="O139" s="17" t="n"/>
+      <c r="P139" s="16" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="16" t="n"/>
@@ -5116,6 +5270,7 @@
       <c r="M140" s="17" t="n"/>
       <c r="N140" s="18" t="n"/>
       <c r="O140" s="17" t="n"/>
+      <c r="P140" s="16" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="16" t="n"/>
@@ -5133,6 +5288,7 @@
       <c r="M141" s="17" t="n"/>
       <c r="N141" s="18" t="n"/>
       <c r="O141" s="17" t="n"/>
+      <c r="P141" s="16" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="16" t="n"/>
@@ -5150,6 +5306,7 @@
       <c r="M142" s="17" t="n"/>
       <c r="N142" s="18" t="n"/>
       <c r="O142" s="17" t="n"/>
+      <c r="P142" s="16" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="16" t="n"/>
@@ -5167,6 +5324,7 @@
       <c r="M143" s="17" t="n"/>
       <c r="N143" s="18" t="n"/>
       <c r="O143" s="17" t="n"/>
+      <c r="P143" s="16" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="16" t="n"/>
@@ -5184,6 +5342,7 @@
       <c r="M144" s="17" t="n"/>
       <c r="N144" s="18" t="n"/>
       <c r="O144" s="17" t="n"/>
+      <c r="P144" s="16" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="16" t="n"/>
@@ -5201,6 +5360,7 @@
       <c r="M145" s="17" t="n"/>
       <c r="N145" s="18" t="n"/>
       <c r="O145" s="17" t="n"/>
+      <c r="P145" s="16" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="16" t="n"/>
@@ -5218,6 +5378,7 @@
       <c r="M146" s="17" t="n"/>
       <c r="N146" s="18" t="n"/>
       <c r="O146" s="17" t="n"/>
+      <c r="P146" s="16" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="16" t="n"/>
@@ -5235,6 +5396,7 @@
       <c r="M147" s="17" t="n"/>
       <c r="N147" s="18" t="n"/>
       <c r="O147" s="17" t="n"/>
+      <c r="P147" s="16" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="16" t="n"/>
@@ -5252,6 +5414,7 @@
       <c r="M148" s="17" t="n"/>
       <c r="N148" s="18" t="n"/>
       <c r="O148" s="17" t="n"/>
+      <c r="P148" s="16" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="16" t="n"/>
@@ -5269,6 +5432,7 @@
       <c r="M149" s="17" t="n"/>
       <c r="N149" s="18" t="n"/>
       <c r="O149" s="17" t="n"/>
+      <c r="P149" s="16" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="16" t="n"/>
@@ -5286,6 +5450,7 @@
       <c r="M150" s="17" t="n"/>
       <c r="N150" s="18" t="n"/>
       <c r="O150" s="17" t="n"/>
+      <c r="P150" s="16" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="16" t="n"/>
@@ -5303,6 +5468,7 @@
       <c r="M151" s="17" t="n"/>
       <c r="N151" s="18" t="n"/>
       <c r="O151" s="17" t="n"/>
+      <c r="P151" s="16" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="16" t="n"/>
@@ -5320,6 +5486,7 @@
       <c r="M152" s="17" t="n"/>
       <c r="N152" s="18" t="n"/>
       <c r="O152" s="17" t="n"/>
+      <c r="P152" s="16" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="16" t="n"/>
@@ -5337,6 +5504,7 @@
       <c r="M153" s="17" t="n"/>
       <c r="N153" s="18" t="n"/>
       <c r="O153" s="17" t="n"/>
+      <c r="P153" s="16" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="16" t="n"/>
@@ -5354,6 +5522,7 @@
       <c r="M154" s="17" t="n"/>
       <c r="N154" s="18" t="n"/>
       <c r="O154" s="17" t="n"/>
+      <c r="P154" s="16" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="16" t="n"/>
@@ -5371,6 +5540,7 @@
       <c r="M155" s="17" t="n"/>
       <c r="N155" s="18" t="n"/>
       <c r="O155" s="17" t="n"/>
+      <c r="P155" s="16" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="16" t="n"/>
@@ -5388,6 +5558,7 @@
       <c r="M156" s="17" t="n"/>
       <c r="N156" s="18" t="n"/>
       <c r="O156" s="17" t="n"/>
+      <c r="P156" s="16" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="16" t="n"/>
@@ -5405,6 +5576,7 @@
       <c r="M157" s="17" t="n"/>
       <c r="N157" s="18" t="n"/>
       <c r="O157" s="17" t="n"/>
+      <c r="P157" s="16" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="16" t="n"/>
@@ -5422,6 +5594,7 @@
       <c r="M158" s="17" t="n"/>
       <c r="N158" s="18" t="n"/>
       <c r="O158" s="17" t="n"/>
+      <c r="P158" s="16" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="16" t="n"/>
@@ -5439,6 +5612,7 @@
       <c r="M159" s="17" t="n"/>
       <c r="N159" s="18" t="n"/>
       <c r="O159" s="17" t="n"/>
+      <c r="P159" s="16" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="16" t="n"/>
@@ -5456,6 +5630,7 @@
       <c r="M160" s="17" t="n"/>
       <c r="N160" s="18" t="n"/>
       <c r="O160" s="17" t="n"/>
+      <c r="P160" s="16" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="16" t="n"/>
@@ -5473,6 +5648,7 @@
       <c r="M161" s="17" t="n"/>
       <c r="N161" s="18" t="n"/>
       <c r="O161" s="17" t="n"/>
+      <c r="P161" s="16" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="16" t="n"/>
@@ -5490,6 +5666,7 @@
       <c r="M162" s="17" t="n"/>
       <c r="N162" s="18" t="n"/>
       <c r="O162" s="17" t="n"/>
+      <c r="P162" s="16" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="16" t="n"/>
@@ -5507,6 +5684,7 @@
       <c r="M163" s="17" t="n"/>
       <c r="N163" s="18" t="n"/>
       <c r="O163" s="17" t="n"/>
+      <c r="P163" s="16" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="16" t="n"/>
@@ -5524,6 +5702,7 @@
       <c r="M164" s="17" t="n"/>
       <c r="N164" s="18" t="n"/>
       <c r="O164" s="17" t="n"/>
+      <c r="P164" s="16" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="16" t="n"/>
@@ -5541,6 +5720,7 @@
       <c r="M165" s="17" t="n"/>
       <c r="N165" s="18" t="n"/>
       <c r="O165" s="17" t="n"/>
+      <c r="P165" s="16" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="16" t="n"/>
@@ -5558,6 +5738,7 @@
       <c r="M166" s="17" t="n"/>
       <c r="N166" s="18" t="n"/>
       <c r="O166" s="17" t="n"/>
+      <c r="P166" s="16" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="16" t="n"/>
@@ -5575,6 +5756,7 @@
       <c r="M167" s="17" t="n"/>
       <c r="N167" s="18" t="n"/>
       <c r="O167" s="17" t="n"/>
+      <c r="P167" s="16" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="16" t="n"/>
@@ -5592,6 +5774,7 @@
       <c r="M168" s="17" t="n"/>
       <c r="N168" s="18" t="n"/>
       <c r="O168" s="17" t="n"/>
+      <c r="P168" s="16" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="16" t="n"/>
@@ -5609,6 +5792,7 @@
       <c r="M169" s="17" t="n"/>
       <c r="N169" s="18" t="n"/>
       <c r="O169" s="17" t="n"/>
+      <c r="P169" s="16" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="16" t="n"/>
@@ -5626,6 +5810,7 @@
       <c r="M170" s="17" t="n"/>
       <c r="N170" s="18" t="n"/>
       <c r="O170" s="17" t="n"/>
+      <c r="P170" s="16" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="16" t="n"/>
@@ -5643,6 +5828,7 @@
       <c r="M171" s="17" t="n"/>
       <c r="N171" s="18" t="n"/>
       <c r="O171" s="17" t="n"/>
+      <c r="P171" s="16" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="16" t="n"/>
@@ -5660,6 +5846,7 @@
       <c r="M172" s="17" t="n"/>
       <c r="N172" s="18" t="n"/>
       <c r="O172" s="17" t="n"/>
+      <c r="P172" s="16" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="16" t="n"/>
@@ -5677,6 +5864,7 @@
       <c r="M173" s="17" t="n"/>
       <c r="N173" s="18" t="n"/>
       <c r="O173" s="17" t="n"/>
+      <c r="P173" s="16" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="16" t="n"/>
@@ -5694,6 +5882,7 @@
       <c r="M174" s="17" t="n"/>
       <c r="N174" s="18" t="n"/>
       <c r="O174" s="17" t="n"/>
+      <c r="P174" s="16" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="16" t="n"/>
@@ -5711,6 +5900,7 @@
       <c r="M175" s="17" t="n"/>
       <c r="N175" s="18" t="n"/>
       <c r="O175" s="17" t="n"/>
+      <c r="P175" s="16" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="16" t="n"/>
@@ -5728,6 +5918,7 @@
       <c r="M176" s="17" t="n"/>
       <c r="N176" s="18" t="n"/>
       <c r="O176" s="17" t="n"/>
+      <c r="P176" s="16" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="16" t="n"/>
@@ -5745,6 +5936,7 @@
       <c r="M177" s="17" t="n"/>
       <c r="N177" s="18" t="n"/>
       <c r="O177" s="17" t="n"/>
+      <c r="P177" s="16" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="16" t="n"/>
@@ -5762,6 +5954,7 @@
       <c r="M178" s="17" t="n"/>
       <c r="N178" s="18" t="n"/>
       <c r="O178" s="17" t="n"/>
+      <c r="P178" s="16" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="16" t="n"/>
@@ -5779,6 +5972,7 @@
       <c r="M179" s="17" t="n"/>
       <c r="N179" s="18" t="n"/>
       <c r="O179" s="17" t="n"/>
+      <c r="P179" s="16" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="16" t="n"/>
@@ -5796,6 +5990,7 @@
       <c r="M180" s="17" t="n"/>
       <c r="N180" s="18" t="n"/>
       <c r="O180" s="17" t="n"/>
+      <c r="P180" s="16" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="16" t="n"/>
@@ -5813,6 +6008,7 @@
       <c r="M181" s="17" t="n"/>
       <c r="N181" s="18" t="n"/>
       <c r="O181" s="17" t="n"/>
+      <c r="P181" s="16" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="16" t="n"/>
@@ -5830,6 +6026,7 @@
       <c r="M182" s="17" t="n"/>
       <c r="N182" s="18" t="n"/>
       <c r="O182" s="17" t="n"/>
+      <c r="P182" s="16" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="16" t="n"/>
@@ -5847,6 +6044,7 @@
       <c r="M183" s="17" t="n"/>
       <c r="N183" s="18" t="n"/>
       <c r="O183" s="17" t="n"/>
+      <c r="P183" s="16" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="16" t="n"/>
@@ -5864,6 +6062,7 @@
       <c r="M184" s="17" t="n"/>
       <c r="N184" s="18" t="n"/>
       <c r="O184" s="17" t="n"/>
+      <c r="P184" s="16" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="16" t="n"/>
@@ -5881,6 +6080,7 @@
       <c r="M185" s="17" t="n"/>
       <c r="N185" s="18" t="n"/>
       <c r="O185" s="17" t="n"/>
+      <c r="P185" s="16" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="16" t="n"/>
@@ -5898,6 +6098,7 @@
       <c r="M186" s="17" t="n"/>
       <c r="N186" s="18" t="n"/>
       <c r="O186" s="17" t="n"/>
+      <c r="P186" s="16" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="16" t="n"/>
@@ -5915,6 +6116,7 @@
       <c r="M187" s="17" t="n"/>
       <c r="N187" s="18" t="n"/>
       <c r="O187" s="17" t="n"/>
+      <c r="P187" s="16" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="16" t="n"/>
@@ -5932,6 +6134,7 @@
       <c r="M188" s="17" t="n"/>
       <c r="N188" s="18" t="n"/>
       <c r="O188" s="17" t="n"/>
+      <c r="P188" s="16" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="16" t="n"/>
@@ -5949,6 +6152,7 @@
       <c r="M189" s="17" t="n"/>
       <c r="N189" s="18" t="n"/>
       <c r="O189" s="17" t="n"/>
+      <c r="P189" s="16" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="16" t="n"/>
@@ -5966,6 +6170,7 @@
       <c r="M190" s="17" t="n"/>
       <c r="N190" s="18" t="n"/>
       <c r="O190" s="17" t="n"/>
+      <c r="P190" s="16" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="16" t="n"/>
@@ -5983,6 +6188,7 @@
       <c r="M191" s="17" t="n"/>
       <c r="N191" s="18" t="n"/>
       <c r="O191" s="17" t="n"/>
+      <c r="P191" s="16" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="16" t="n"/>
@@ -6000,6 +6206,7 @@
       <c r="M192" s="17" t="n"/>
       <c r="N192" s="18" t="n"/>
       <c r="O192" s="17" t="n"/>
+      <c r="P192" s="16" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="16" t="n"/>
@@ -6017,6 +6224,7 @@
       <c r="M193" s="17" t="n"/>
       <c r="N193" s="18" t="n"/>
       <c r="O193" s="17" t="n"/>
+      <c r="P193" s="16" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="16" t="n"/>
@@ -6034,6 +6242,7 @@
       <c r="M194" s="17" t="n"/>
       <c r="N194" s="18" t="n"/>
       <c r="O194" s="17" t="n"/>
+      <c r="P194" s="16" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="16" t="n"/>
@@ -6051,6 +6260,7 @@
       <c r="M195" s="17" t="n"/>
       <c r="N195" s="18" t="n"/>
       <c r="O195" s="17" t="n"/>
+      <c r="P195" s="16" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="16" t="n"/>
@@ -6068,6 +6278,7 @@
       <c r="M196" s="17" t="n"/>
       <c r="N196" s="18" t="n"/>
       <c r="O196" s="17" t="n"/>
+      <c r="P196" s="16" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="16" t="n"/>
@@ -6085,6 +6296,7 @@
       <c r="M197" s="17" t="n"/>
       <c r="N197" s="18" t="n"/>
       <c r="O197" s="17" t="n"/>
+      <c r="P197" s="16" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="16" t="n"/>
@@ -6102,6 +6314,7 @@
       <c r="M198" s="17" t="n"/>
       <c r="N198" s="18" t="n"/>
       <c r="O198" s="17" t="n"/>
+      <c r="P198" s="16" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="16" t="n"/>
@@ -6119,6 +6332,7 @@
       <c r="M199" s="17" t="n"/>
       <c r="N199" s="18" t="n"/>
       <c r="O199" s="17" t="n"/>
+      <c r="P199" s="16" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="16" t="n"/>
@@ -6136,6 +6350,7 @@
       <c r="M200" s="17" t="n"/>
       <c r="N200" s="18" t="n"/>
       <c r="O200" s="17" t="n"/>
+      <c r="P200" s="16" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="16" t="n"/>
@@ -6153,6 +6368,7 @@
       <c r="M201" s="17" t="n"/>
       <c r="N201" s="18" t="n"/>
       <c r="O201" s="17" t="n"/>
+      <c r="P201" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O201"/>

</xml_diff>